<commit_message>
Persist dashboard edit defaults
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -2,43 +2,29 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="4480" yWindow="500" windowWidth="33600" windowHeight="20500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标说明" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'指标说明'!$A$1:$C$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'指标说明'!$A$1:$C$65</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <sz val="9"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -46,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -55,61 +41,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF2F8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEAF7EF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF4E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2ECF9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EAF2F8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EAF7EF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF4E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2ECF9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -117,83 +53,21 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFD9E2F3"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFD9E2F3"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFD9E2F3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFD9E2F3"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D9E2F3"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D9E2F3"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D9E2F3"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9E2F3"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -556,1168 +430,1121 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C68"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <dimension ref="A1:C65"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="86" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>模块</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>指标</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>指标定义</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>UV (独立访客)</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>独立访客数</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>PV (页面浏览量)</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>页面浏览量</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>人均停留时长</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>人均会话停留时长</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>整体跳出率</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>单页访问即离开比例</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>招募单点击率</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>招募卡片点击占曝光比例</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>招募搜索次数</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>招募单搜索提交次数</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>招募单搜索次数</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>招募单名称搜索提交次数</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>流量来源分布</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>各来源 UV/PV 占比</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>受访页面排行</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>页面 PV/UV 排名</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>新老访客比例</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>时间范围内新访客和老访客分别占全部独立访客的比例</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>设备终端分布</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>PC/移动/平板访问比例</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>平台流量</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>招募卡片点击量</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>招募卡片被点击的次数</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>注册总用户数</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>平台累计注册众包用户数</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>今日新增注册</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>时间范围内新增注册用户</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>DAU 今日活跃</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>当日活跃用户</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>MAU 月活用户</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>近 30 天或自然月活跃用户</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>平台活跃率</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>平台月活跃用户占比</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>月活占注册用户比例</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>注册转化率</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>新访客注册转化率</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>访客转注册比例</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>实名认证率</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>已实名认证用户占比</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>招募申请率</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>认证后提交申请比例</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>90天未活跃用户</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>统计日内首次达到连续 90 天无登录且无有效任务行为的用户数</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="48" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>转化环节流失率</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>用户转化漏斗中，指定环节未进入下一阶段的人数占进入该环节人数的比例；不等同于 90 天未活跃/已流失用户</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="48" customHeight="1">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>新注册用户</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>入组时间范围内完成注册的去重用户数，是 D30 转化漏斗分母</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>完成实名认证</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>新注册 cohort 中，注册后 30 天内完成实名认证的用户数</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="48" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>提交招募申请</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>新注册 cohort 中，注册后 30 天内至少提交过一次招募申请的用户数</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="48" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>招募通过</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>新注册 cohort 中，注册后 30 天内至少有一个招募申请审核通过的用户数</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="48" customHeight="1">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>参与任务执行</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>新注册 cohort 中，注册后 30 天内产生首次有效任务行为的用户数</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="48" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>D30持续活跃 Worker</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>新注册 cohort 中，注册后第 24-30 天仍有有效任务提交的用户数</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="48" customHeight="1">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>环节转化</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>当前阶段人数占上一阶段人数的比例</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="48" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>累计转化</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>当前阶段人数占新注册用户人数的比例</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="48" customHeight="1">
-      <c r="A31" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>较上一步流失</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>上一阶段进入人数与当前阶段人数的差值</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="48" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>用户数</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>指定注册周期内的注册用户数</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="48" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>D1 留存</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>cohort 注册后第 1 天活跃比例</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="48" customHeight="1">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>D7 留存</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>cohort 注册后第 7 天活跃比例</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="48" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>D14 留存</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>cohort 注册后第 14 天活跃比例</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="48" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>D30 留存</t>
         </is>
       </c>
-      <c r="C36" s="9" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>cohort 注册后第 30 天活跃比例</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="48" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>生命周期阶段人数</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>按用户当前生命周期状态归类的用户数；已流失阶段指连续 90 天无登录且无有效任务行为的用户</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="48" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>已流失用户</t>
         </is>
       </c>
-      <c r="C38" s="9" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>截至统计日，连续 90 天无登录且无有效任务行为的用户数；重新登录或产生有效任务行为后退出已流失状态</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="48" customHeight="1">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>平均生命周期</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>注册到已流失判定日的平均天数；未达到已流失状态的用户统计到当前日期，已流失按连续 90 天无登录且无有效任务行为判定</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="48" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B40" s="9" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>注册→首单</t>
         </is>
       </c>
-      <c r="C40" s="9" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>注册到首次参与任务的时长</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="48" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B41" s="9" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>生命周期时长分布</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>按用户生命周期时长区间统计的用户占比</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="48" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B42" s="9" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>新增招募单</t>
         </is>
       </c>
-      <c r="C42" s="9" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>时间范围内创建的招募单数</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="48" customHeight="1">
-      <c r="A43" s="11" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>进行中招募单</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>状态为招募中或可接收申请的招募单</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="48" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>已完成招募单</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>状态为已完成的招募单</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="48" customHeight="1">
-      <c r="A45" s="11" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B45" s="9" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>目标招募总人数 / 目标人数</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>招募单目标人数</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="48" customHeight="1">
-      <c r="A46" s="11" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>已到位总人数</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
-        <is>
-          <t>通过并参与任务或自动加入任务的人数</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="48" customHeight="1">
-      <c r="A47" s="11" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>招募通过总人数 / 招募通过人数</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>招募申请审核通过的去重人数</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>总缺口人数 / 缺口人数</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
-        <is>
-          <t>未满足目标的人数</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="48" customHeight="1">
-      <c r="A48" s="11" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>目标人数与招募通过人数之间的差额</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B48" s="9" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>缺口率</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
-        <is>
-          <t>缺口占目标比例</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="48" customHeight="1">
-      <c r="A49" s="11" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>缺口人数占目标人数比例</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B49" s="9" t="inlineStr">
-        <is>
-          <t>招募供需缺口</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
-        <is>
-          <t>目标人数与已到位人数差额</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="48" customHeight="1">
-      <c r="A50" s="11" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>通过率 / 整体通过率</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>审批通过申请占已审核申请比例</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>通过率 / 整体通过率</t>
-        </is>
-      </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>审批通过比例</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="48" customHeight="1">
-      <c r="A51" s="11" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>申请率</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>访问或曝光后提交申请比例</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>招募通过率</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>审批通过申请占比</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="48" customHeight="1">
-      <c r="A52" s="11" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>招募单数</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>按业务领域统计的招募单数量</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B52" s="9" t="inlineStr">
-        <is>
-          <t>申请率</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>访问/曝光后提交申请比例</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="48" customHeight="1">
-      <c r="A53" s="11" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>申请人数</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>提交过申请的人数</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B53" s="9" t="inlineStr">
-        <is>
-          <t>招募单数</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>按业务领域统计的招募单数量</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="48" customHeight="1">
-      <c r="A54" s="11" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>平均审核周期</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>申请到审批完成平均时长</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B54" s="9" t="inlineStr">
-        <is>
-          <t>申请人数</t>
-        </is>
-      </c>
-      <c r="C54" s="9" t="inlineStr">
-        <is>
-          <t>提交过申请的人数</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="48" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B55" s="9" t="inlineStr">
-        <is>
-          <t>招募通过人数</t>
-        </is>
-      </c>
-      <c r="C55" s="9" t="inlineStr">
-        <is>
-          <t>招募申请审核通过的去重人数</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="48" customHeight="1">
-      <c r="A56" s="11" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B56" s="9" t="inlineStr">
-        <is>
-          <t>平均审核周期</t>
-        </is>
-      </c>
-      <c r="C56" s="9" t="inlineStr">
-        <is>
-          <t>申请到审批完成平均时长</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="48" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B57" s="9" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>通过达成率</t>
         </is>
       </c>
-      <c r="C57" s="9" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>招募通过人数占目标招募人数的比例</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="48" customHeight="1">
-      <c r="A58" s="12" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B58" s="9" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>进行中任务数</t>
         </is>
       </c>
-      <c r="C58" s="9" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>当前进行中任务数量</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="48" customHeight="1">
-      <c r="A59" s="12" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B59" s="9" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>参与人数</t>
         </is>
       </c>
-      <c r="C59" s="9" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>时间范围内参与任务人数</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="48" customHeight="1">
-      <c r="A60" s="12" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B60" s="9" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>总提交量</t>
         </is>
       </c>
-      <c r="C60" s="9" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>时间范围内提交条数</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="48" customHeight="1">
-      <c r="A61" s="12" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B61" s="9" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>今日提交量</t>
         </is>
       </c>
-      <c r="C61" s="9" t="inlineStr">
+      <c r="C57" s="2" t="inlineStr">
         <is>
           <t>当日提交条数</t>
         </is>
       </c>
     </row>
-    <row r="62" ht="48" customHeight="1">
-      <c r="A62" s="12" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B62" s="9" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>今日提交数据</t>
         </is>
       </c>
-      <c r="C62" s="9" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>当日提交数据条数</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="48" customHeight="1">
-      <c r="A63" s="12" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B63" s="9" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>人均日产能</t>
         </is>
       </c>
-      <c r="C63" s="9" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>每活跃人员日均提交条数</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="48" customHeight="1">
-      <c r="A64" s="12" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B64" s="9" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>标注提交数据条数</t>
         </is>
       </c>
-      <c r="C64" s="9" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>时间范围内标注任务提交的数据条数</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="48" customHeight="1">
-      <c r="A65" s="12" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B65" s="9" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>采集提交数据条数</t>
         </is>
       </c>
-      <c r="C65" s="9" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>时间范围内采集任务提交的数据条数</t>
         </is>
       </c>
     </row>
-    <row r="66" ht="48" customHeight="1">
-      <c r="A66" s="12" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B66" s="9" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>标注质检通过率</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>标注任务通过质检的数据占标注任务已质检数据的比例</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>任务&amp;质量</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>采集质检通过率</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>采集任务通过质检的数据占采集任务已质检数据的比例</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>任务&amp;质量</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>后续质检通过率</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
-        <is>
-          <t>标注（采集）提交条数/标注（采集）提交次数</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="48" customHeight="1">
-      <c r="A67" s="12" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>首次质检未通过后，进入后续质检并通过的数据占比，不拆分具体轮次</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B67" s="9" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>错误类型占比</t>
         </is>
       </c>
-      <c r="C67" s="9" t="inlineStr">
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>各错误类型占质检错误比例</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="48" customHeight="1">
-      <c r="A68" s="13" t="n"/>
-      <c r="B68" s="9" t="n"/>
-      <c r="C68" s="9" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:C68"/>
+  <autoFilter ref="A1:C65"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;L&amp;"Calibri"&amp;10 &amp;K000000_x000d_# This content is for internal use only</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Align recruit pass rate metric
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -1330,12 +1330,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>通过达成率</t>
+          <t>通过率</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>招募通过人数占目标招募人数的比例</t>
+          <t>审批通过申请占已审核申请比例</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify D30 funnel active metric
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -918,7 +918,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>以统计日前 31-60 天完成注册的用户作为入组用户，观察注册后 0-30 天内提交招募申请、招募通过、参与任务执行和 D30 持续活跃的达成人数。</t>
+          <t>以统计日前 31-60 天完成注册的用户作为入组用户，确保每个入组用户都已完整经历注册后 0-30 天观察期；展示其在提交招募申请、招募通过、参与任务执行和 D30窗口活跃等关键阶段的达成人数。</t>
         </is>
       </c>
     </row>
@@ -998,12 +998,12 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>D30持续活跃用户</t>
+          <t>D30窗口活跃用户</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>新注册用户分组中，注册后第 24-30 天仍有有效任务提交的用户数，用于衡量首单后留存。</t>
+          <t>已完整经历 30 天观察期的新注册用户中，注册后第 24-30 天内至少有一次有效任务提交的用户数；未注册满 30 天的新用户不纳入统计。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix tooltips and clarify churn breakpoint
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1338,12 +1338,12 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>用户流失原因分析</t>
+          <t>转化流失断点分析</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>按转化环节展示进入该环节后未进入下一环节的流失人数和流失率，不等同于 90 天未活跃/已流失用户。</t>
+          <t>按相邻转化环节展示进入该环节后未进入下一环节的流失人数和流失率，用于定位转化阻塞点；不等同于 90 天未活跃/已流失用户。</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>用户转化漏斗中进入指定环节后未进入下一环节的去重用户数；不用于用户增长趋势中的 90 天未活跃用户口径。</t>
+          <t>用户转化漏斗中进入指定环节后未进入下一环节的去重用户数；与转化环节流失率使用同一批进入该环节的用户作为基准。</t>
         </is>
       </c>
     </row>
@@ -1377,24 +1377,24 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数；不等同于 90 天未活跃/已流失用户。</t>
+          <t>进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数；用于比较相邻转化断点，不应对多个环节简单平均，不等同于 90 天未活跃/已流失用户。</t>
         </is>
       </c>
     </row>
     <row r="53" ht="52" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>用户平均生命周期时长</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>观察用户从注册到流失或当前日期的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>最大流失断点</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>转化流失断点分析中流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位当前最明显的转化阻塞点。</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1406,12 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>平均生命周期</t>
+          <t>用户平均生命周期时长</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>纳入样本用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到当前日期，已流失按连续 90 天无登录且无有效任务行为判定。</t>
+          <t>观察用户从注册到流失或当前日期的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
         </is>
       </c>
     </row>
@@ -1423,12 +1423,12 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>注册→首单</t>
+          <t>平均生命周期</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
+          <t>纳入样本用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到当前日期，已流失按连续 90 天无登录且无有效任务行为判定。</t>
         </is>
       </c>
     </row>
@@ -1440,29 +1440,29 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
+          <t>注册→首单</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="52" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
           <t>生命周期时长分布</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到当前日期。</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="52" customHeight="1">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>新增招募单</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
-        <is>
-          <t>所选时间范围内新创建的招募单数量，按招募单 ID 去重。</t>
         </is>
       </c>
     </row>
@@ -1474,12 +1474,12 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>进行中招募单</t>
+          <t>新增招募单</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>截至统计日状态为招募中，且仍可接收用户申请的招募单数量，按招募单 ID 去重。</t>
+          <t>所选时间范围内新创建的招募单数量，按招募单 ID 去重。</t>
         </is>
       </c>
     </row>
@@ -1491,12 +1491,12 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>已完成招募单</t>
+          <t>进行中招募单</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>所选时间范围内状态为已完成的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成。</t>
+          <t>截至统计日状态为招募中，且仍可接收用户申请的招募单数量，按招募单 ID 去重。</t>
         </is>
       </c>
     </row>
@@ -1508,12 +1508,12 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>目标招募总人数</t>
+          <t>已完成招募单</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>所选招募单计划招募人数的合计，按招募单目标人数汇总。</t>
+          <t>所选时间范围内状态为已完成的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成。</t>
         </is>
       </c>
     </row>
@@ -1525,12 +1525,12 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>招募通过总人数</t>
+          <t>目标招募总人数</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>所选范围内招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；不等同于已到位人数。</t>
+          <t>所选招募单计划招募人数的合计，按招募单目标人数汇总。</t>
         </is>
       </c>
     </row>
@@ -1542,12 +1542,12 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>总缺口人数</t>
+          <t>招募通过总人数</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
+          <t>所选范围内招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；不等同于已到位人数。</t>
         </is>
       </c>
     </row>
@@ -1559,12 +1559,12 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>整体通过率</t>
+          <t>总缺口人数</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
+          <t>目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
         </is>
       </c>
     </row>
@@ -1576,12 +1576,12 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>招募转化趋势</t>
+          <t>整体通过率</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>按日期展示申请率和通过率趋势；申请率为提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数，通过率为审核通过的招募申请数/已完成审核的招募申请数。</t>
+          <t>审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
         </is>
       </c>
     </row>
@@ -1593,12 +1593,12 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>申请率</t>
+          <t>招募转化趋势</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数。</t>
+          <t>按日期展示申请率和通过率趋势；申请率为提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数，通过率为审核通过的招募申请数/已完成审核的招募申请数。</t>
         </is>
       </c>
     </row>
@@ -1610,12 +1610,12 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>通过率</t>
+          <t>申请率</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
+          <t>提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1627,12 +1627,12 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>招募单数</t>
+          <t>通过率</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>所选范围内招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量。</t>
+          <t>审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
         </is>
       </c>
     </row>
@@ -1644,12 +1644,12 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>目标人数</t>
+          <t>招募单数</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>所选招募单计划招募人数的合计，按招募单目标人数汇总。</t>
+          <t>所选范围内招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量。</t>
         </is>
       </c>
     </row>
@@ -1661,12 +1661,12 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>申请人数</t>
+          <t>目标人数</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>所选范围内提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次。</t>
+          <t>所选招募单计划招募人数的合计，按招募单目标人数汇总。</t>
         </is>
       </c>
     </row>
@@ -1678,12 +1678,12 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>招募通过人数</t>
+          <t>申请人数</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>所选范围内招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；不等同于已到位人数。</t>
+          <t>所选范围内提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次。</t>
         </is>
       </c>
     </row>
@@ -1695,12 +1695,12 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>缺口人数</t>
+          <t>招募通过人数</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
+          <t>所选范围内招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；不等同于已到位人数。</t>
         </is>
       </c>
     </row>
@@ -1712,12 +1712,12 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>缺口率</t>
+          <t>缺口人数</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>缺口人数/目标招募人数；目标人数为 0 时不计算。</t>
+          <t>目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
         </is>
       </c>
     </row>
@@ -1729,12 +1729,12 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>平均审核周期</t>
+          <t>缺口率</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计。</t>
+          <t>缺口人数/目标招募人数；目标人数为 0 时不计算。</t>
         </is>
       </c>
     </row>
@@ -1746,29 +1746,29 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
+          <t>平均审核周期</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="52" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>招募分析</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
           <t>明细招募单状态</t>
         </is>
       </c>
-      <c r="C74" s="7" t="inlineStr">
+      <c r="C75" s="7" t="inlineStr">
         <is>
           <t>明细招募单当前状态，包含招募中、审核中、已暂停、已完成，用于配合招募单状态筛选查看不同状态下的招募表现。</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="52" customHeight="1">
-      <c r="A75" s="8" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B75" s="8" t="inlineStr">
-        <is>
-          <t>进行中任务数</t>
-        </is>
-      </c>
-      <c r="C75" s="9" t="inlineStr">
-        <is>
-          <t>截至统计日状态为进行中且可被执行或提交的任务数量，按任务 ID 去重。</t>
         </is>
       </c>
     </row>
@@ -1780,12 +1780,12 @@
       </c>
       <c r="B76" s="8" t="inlineStr">
         <is>
-          <t>参与人数</t>
+          <t>进行中任务数</t>
         </is>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>所选时间范围内产生领取、进入任务、提交或质检相关有效任务行为的去重用户数。</t>
+          <t>截至统计日状态为进行中且可被执行或提交的任务数量，按任务 ID 去重。</t>
         </is>
       </c>
     </row>
@@ -1797,12 +1797,12 @@
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>总提交量</t>
+          <t>参与人数</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>所选时间范围内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
+          <t>所选时间范围内产生领取、进入任务、提交或质检相关有效任务行为的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1814,12 +1814,12 @@
       </c>
       <c r="B78" s="8" t="inlineStr">
         <is>
-          <t>标注质检通过率</t>
+          <t>总提交量</t>
         </is>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>标注任务中质检通过的数据条数/标注任务中已完成质检的数据条数。</t>
+          <t>所选时间范围内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
         </is>
       </c>
     </row>
@@ -1831,12 +1831,12 @@
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>今日提交量</t>
+          <t>标注质检通过率</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>统计日内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
+          <t>标注任务中质检通过的数据条数/标注任务中已完成质检的数据条数。</t>
         </is>
       </c>
     </row>
@@ -1848,12 +1848,12 @@
       </c>
       <c r="B80" s="8" t="inlineStr">
         <is>
-          <t>人均日产能</t>
+          <t>今日提交量</t>
         </is>
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>统计日任务提交数据条数/统计日有有效任务行为的去重用户数。</t>
+          <t>统计日内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
         </is>
       </c>
     </row>
@@ -1865,12 +1865,12 @@
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>采集质检通过率</t>
+          <t>人均日产能</t>
         </is>
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>采集任务中质检通过的数据条数/采集任务中已完成质检的数据条数。</t>
+          <t>统计日任务提交数据条数/统计日有有效任务行为的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1882,12 +1882,12 @@
       </c>
       <c r="B82" s="8" t="inlineStr">
         <is>
-          <t>数据产出趋势</t>
+          <t>采集质检通过率</t>
         </is>
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>按日期展示标注提交数据条数和采集提交数据条数，用于观察不同任务类型的数据产出变化。</t>
+          <t>采集任务中质检通过的数据条数/采集任务中已完成质检的数据条数。</t>
         </is>
       </c>
     </row>
@@ -1899,12 +1899,12 @@
       </c>
       <c r="B83" s="8" t="inlineStr">
         <is>
-          <t>标注提交数据条数</t>
+          <t>数据产出趋势</t>
         </is>
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>所选时间范围内标注任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
+          <t>按日期展示标注提交数据条数和采集提交数据条数，用于观察不同任务类型的数据产出变化。</t>
         </is>
       </c>
     </row>
@@ -1916,12 +1916,12 @@
       </c>
       <c r="B84" s="8" t="inlineStr">
         <is>
-          <t>采集提交数据条数</t>
+          <t>标注提交数据条数</t>
         </is>
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>所选时间范围内采集任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
+          <t>所选时间范围内标注任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
         </is>
       </c>
     </row>
@@ -1933,12 +1933,12 @@
       </c>
       <c r="B85" s="8" t="inlineStr">
         <is>
-          <t>后续质检通过率趋势</t>
+          <t>采集提交数据条数</t>
         </is>
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>按日期展示后续质检通过率；后续质检通过率为首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数，不拆分具体轮次。</t>
+          <t>所选时间范围内采集任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
         </is>
       </c>
     </row>
@@ -1950,12 +1950,12 @@
       </c>
       <c r="B86" s="8" t="inlineStr">
         <is>
-          <t>后续质检通过率</t>
+          <t>后续质检通过率趋势</t>
         </is>
       </c>
       <c r="C86" s="9" t="inlineStr">
         <is>
-          <t>首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数；不拆分具体轮次。</t>
+          <t>按日期展示后续质检通过率；后续质检通过率为首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数，不拆分具体轮次。</t>
         </is>
       </c>
     </row>
@@ -1967,12 +1967,12 @@
       </c>
       <c r="B87" s="8" t="inlineStr">
         <is>
-          <t>错误类型分布</t>
+          <t>后续质检通过率</t>
         </is>
       </c>
       <c r="C87" s="9" t="inlineStr">
         <is>
-          <t>按错误类型展示质检错误结构，错误类型占比为指定错误类型的错误条数/全部质检错误条数。</t>
+          <t>首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数；不拆分具体轮次。</t>
         </is>
       </c>
     </row>
@@ -1984,12 +1984,12 @@
       </c>
       <c r="B88" s="8" t="inlineStr">
         <is>
-          <t>错误类型占比</t>
+          <t>错误类型分布</t>
         </is>
       </c>
       <c r="C88" s="9" t="inlineStr">
         <is>
-          <t>指定错误类型的错误条数/全部质检错误条数，用于观察错误结构。</t>
+          <t>按错误类型展示质检错误结构，错误类型占比为指定错误类型的错误条数/全部质检错误条数。</t>
         </is>
       </c>
     </row>
@@ -2001,10 +2001,27 @@
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
+          <t>错误类型占比</t>
+        </is>
+      </c>
+      <c r="C89" s="9" t="inlineStr">
+        <is>
+          <t>指定错误类型的错误条数/全部质检错误条数，用于观察错误结构。</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="8" t="inlineStr">
+        <is>
+          <t>任务&amp;质量</t>
+        </is>
+      </c>
+      <c r="B90" s="8" t="inlineStr">
+        <is>
           <t>新用户错误占比</t>
         </is>
       </c>
-      <c r="C89" s="9" t="inlineStr">
+      <c r="C90" s="9" t="inlineStr">
         <is>
           <t>新用户产生的质检错误条数/全部质检错误条数；新用户口径需按平台注册或首单时间窗统一定义。</t>
         </is>

</xml_diff>

<commit_message>
Simplify new user funnel and link retention
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -913,12 +913,12 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>新增用户 D30 转化漏斗</t>
+          <t>新用户转化漏斗（截至当前）</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>以统计日前 31-60 天完成注册的用户作为入组用户，确保每个入组用户都已完整经历注册后 0-30 天观察期；展示其在提交招募申请、招募通过、参与任务执行和 D30窗口活跃等关键阶段的达成人数。</t>
+          <t>按留存矩阵中选中的注册周期展示该批新用户截至当前到达各转化阶段的人数，包括完成实名认证、提交招募申请、招募通过和首次任务执行；用于观察最新转化进度，不强制限定注册后 30 天。</t>
         </is>
       </c>
     </row>
@@ -935,24 +935,24 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>统计日前 31-60 天完成注册的去重用户数，是 D30 转化漏斗的基准用户数；该注册用户分组已完整经过注册后 0-30 天观察窗口。</t>
+          <t>所选注册周期内完成注册的去重用户数，是新用户转化漏斗和留存矩阵联动分析的基准用户数。</t>
         </is>
       </c>
     </row>
     <row r="27" ht="52" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>提交招募申请</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>新注册用户分组中，注册后 30 天内至少提交过一次招募申请的用户数。</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>完成实名认证</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>所选注册周期用户中，截至当前已完成实名认证的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -964,12 +964,12 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>招募通过</t>
+          <t>提交招募申请</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>新注册用户分组中，注册后 30 天内至少有一个招募申请审核通过的用户数。</t>
+          <t>所选注册周期用户中，截至当前至少提交过一次招募申请的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -981,12 +981,12 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>参与任务执行</t>
+          <t>招募通过</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>新注册用户分组中，注册后 30 天内产生首次有效任务行为的用户数，有效任务行为可按领取、进入任务或首次提交定义。</t>
+          <t>所选注册周期用户中，截至当前至少有一个招募申请审核通过的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -998,12 +998,12 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>D30窗口活跃用户</t>
+          <t>首次任务执行</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>已完整经历 30 天观察期的新注册用户中，注册后第 24-30 天内至少有一次有效任务提交的用户数；未注册满 30 天的新用户不纳入统计。</t>
+          <t>所选注册周期用户中，截至当前已产生首次有效任务行为的去重用户数；有效任务行为建议优先使用首次有效任务提交。</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>按注册周期分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率。</t>
+          <t>按注册周期分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率；点击某一注册周期可同步查看该批新用户截至当前的转化漏斗。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove recruitment time filter and update metric docs
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -2,38 +2,52 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="780" yWindow="500" windowWidth="32820" windowHeight="20500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标说明" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'指标说明'!$A$1:$C$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'指标说明'!$A$1:$C$92</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <b val="1"/>
-      <color rgb="000F172A"/>
+      <color rgb="FF0F172A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
+      <sz val="9"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -45,27 +59,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F766E"/>
+        <fgColor rgb="FF0F766E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ECFDF5"/>
+        <fgColor rgb="FFECFDF5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0FDF4"/>
+        <fgColor rgb="FFF0FDF4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0FDFA"/>
+        <fgColor rgb="FFF0FDFA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
+        <fgColor rgb="FFF8FAFC"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,17 +93,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9E2E7"/>
+        <color rgb="FFD9E2E7"/>
       </left>
       <right style="thin">
-        <color rgb="00D9E2E7"/>
+        <color rgb="FFD9E2E7"/>
       </right>
       <top style="thin">
-        <color rgb="00D9E2E7"/>
+        <color rgb="FFD9E2E7"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9E2E7"/>
+        <color rgb="FFD9E2E7"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -126,7 +141,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -489,8 +504,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C90"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C92"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
@@ -527,7 +542,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内访问平台的去重访客数，未登录按访客 ID 去重，已登录按用户 ID 去重。</t>
+          <t>所选统计时间内访问平台的去重访客数，未登录按访客 ID 去重，已登录按用户 ID 去重；可按设备端筛选总计、App 或 Web。</t>
         </is>
       </c>
     </row>
@@ -544,7 +559,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内页面浏览事件次数，同一访客多次浏览累计计数。</t>
+          <t>所选统计时间内页面浏览事件次数，同一访客多次浏览累计计数；可按设备端筛选总计、App 或 Web。</t>
         </is>
       </c>
     </row>
@@ -561,7 +576,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内总会话停留时长除以会话数，异常超长会话按约定上限截断。</t>
+          <t>所选统计时间内总会话停留时长除以会话数，异常超长会话按约定上限截断；可按设备端筛选总计、App 或 Web。</t>
         </is>
       </c>
     </row>
@@ -578,7 +593,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>仅浏览一个页面且未产生有效互动即离开的会话数/进入页面的总会话数。</t>
+          <t>仅浏览一个页面且未产生有效互动即离开的会话数/进入页面的总会话数；可按设备端筛选总计、App 或 Web。</t>
         </is>
       </c>
     </row>
@@ -595,7 +610,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>招募卡片点击次数/招募卡片曝光次数，用于衡量招募单从曝光到点击的转化。</t>
+          <t>招募卡片点击次数/招募卡片曝光次数，用于衡量招募单从曝光到点击的转化；可按设备端筛选总计、App 或 Web。</t>
         </is>
       </c>
     </row>
@@ -607,12 +622,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>招募单搜索次数</t>
+          <t>招募频道点击</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内用户提交招募单搜索的次数，同一用户多次搜索累计计数。</t>
+          <t>所选统计时间内用户点击招募频道标签的次数，同一用户多次点击累计计数；可按设备端筛选总计、App 或 Web。</t>
         </is>
       </c>
     </row>
@@ -624,12 +639,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>流量趋势分析</t>
+          <t>招募单搜索次数</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>按日期展示 PV、UV 与跳出率趋势；PV 为页面浏览事件次数，UV 为去重访客数，跳出率为单页无互动离开会话数/进入页面总会话数。</t>
+          <t>所选统计时间内用户提交招募单搜索的次数，同一用户多次搜索累计计数；可按设备端筛选总计、App 或 Web。</t>
         </is>
       </c>
     </row>
@@ -641,12 +656,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>流量来源占比</t>
+          <t>登录意向点击</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>指定来源带来的 UV 或 PV/全部来源带来的 UV 或 PV，图表展示直接访问、搜索、外链、社媒、邮件等来源结构。</t>
+          <t>所选统计时间内用户点击登录入口，或因访问受保护入口触发登录的次数；可按设备端筛选总计、App 或 Web。</t>
         </is>
       </c>
     </row>
@@ -658,12 +673,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>受访页面排行</t>
+          <t>流量趋势分析</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>按页面维度汇总 PV、UV、平均停留和跳出率，并按浏览量或运营选择的指标排序。</t>
+          <t>按所选统计时间展示 PV、UV 趋势；PV 为页面浏览事件次数，UV 为去重访客数，可按设备端筛选总计、App 或 Web。</t>
         </is>
       </c>
     </row>
@@ -675,12 +690,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>新老访客比例</t>
+          <t>流量来源分布</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>新访客 UV/所选时间范围内全部访问 UV，老访客 UV/所选时间范围内全部访问 UV。</t>
+          <t>按来源展示访问规模和占比；来源访问 UV 或 PV/全部来源访问 UV 或 PV，用于观察直接访问、搜索、外链、社媒、邮件等来源结构。</t>
         </is>
       </c>
     </row>
@@ -692,12 +707,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>设备终端分布</t>
+          <t>受访页面排行</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>指定设备类型访问 UV/全部设备类型访问 UV，用于观察 PC、移动端和平板占比。</t>
+          <t>按页面维度汇总 PV、UV、平均停留和跳出率，并按浏览量或运营选择的指标排序。</t>
         </is>
       </c>
     </row>
@@ -709,12 +724,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>各领域招募单访问情况</t>
+          <t>新老访客比例</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>按业务领域汇总招募单相关 PV 和 UV，用于比较不同领域招募内容获得的访问规模。</t>
+          <t>新访客 UV/所选统计时间内全部访问 UV，老访客 UV/所选统计时间内全部访问 UV。</t>
         </is>
       </c>
     </row>
@@ -726,12 +741,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>招募单访问情况 TOP10</t>
+          <t>设备终端分布</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>按招募单维度展示 PV、UV、招募卡片点击量和点击率；点击率为招募卡片点击次数/招募卡片曝光次数。</t>
+          <t>指定设备端访问 UV/全部设备端访问 UV，用于观察 App 和 Web 的访问占比。</t>
         </is>
       </c>
     </row>
@@ -743,1292 +758,1334 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>各领域招募单访问情况</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>按业务领域汇总招募单相关 PV 和 UV，用于比较不同领域招募内容获得的访问规模。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>平台流量</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>招募单访问情况 TOP10</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>按招募单维度展示 PV、UV、招募卡片点击量和点击率；点击率为招募卡片点击次数/招募卡片曝光次数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>平台流量</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
           <t>招募卡片点击量</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>所选时间范围内招募卡片被点击的次数，同一用户多次点击累计计数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="52" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内招募卡片被点击的次数，同一用户多次点击累计计数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>注册总用户数</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>截至统计日平台累计完成注册的去重众包用户数，以用户 ID 去重。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="52" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>今日新增注册</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>所选时间范围内完成注册的去重用户数，以用户 ID 去重；今日口径按自然日统计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="52" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>DAU 今日活跃</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>统计日内至少发生一次登录、访问核心页面或有效任务行为的去重用户数。</t>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>截至所选统计期末，平台累计完成注册的去重众包用户数，以用户 ID 去重。</t>
         </is>
       </c>
     </row>
     <row r="19" ht="52" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>新增注册</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内完成注册的去重用户数，以用户 ID 去重；选择日时展示单日数据，选择周、月或近 N 天时展示区间汇总数据。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="52" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>DAU 活跃</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>所选统计日期内至少发生一次登录、访问核心页面或有效任务行为的去重用户数；选择周、月或近 N 天时可按区间口径汇总展示。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>MAU 月活用户</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>近 30 天或自然月内至少发生一次登录、访问核心页面或有效任务行为的去重用户数。</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="52" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
+    <row r="22" ht="52" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>平台月活跃用户占比</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>近 30 天或自然月活跃用户数/截至统计日注册总用户数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="52" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>近 30 天或自然月活跃用户数/截至所选统计期末的注册总用户数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="52" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>新访客注册转化率</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>所选时间范围内完成注册的新访客数/同一时间范围内首次访问平台的新访客数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="52" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内完成注册的新访客数/同一统计时间内首次访问平台的新访客数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="52" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>实名认证率</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>已完成实名认证的注册用户数/具备实名认证资格的注册用户数；未开始认证和认证失败均不计入已认证用户数。</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="52" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
+    <row r="25" ht="52" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>招募申请率</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>完成实名认证后提交过至少一次招募申请的用户数/完成实名认证且可申请招募的用户数。</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="52" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
+    <row r="26" ht="52" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>用户增长趋势</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>按日期展示新增注册、活跃用户和 90 天未活跃用户；90 天未活跃用户为统计日当天首次达到连续 90 天无登录且无有效任务行为的去重用户数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="52" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>新用户转化漏斗（截至当前）</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>按留存矩阵中选中的注册周期展示该批新用户截至当前到达各转化阶段的人数，包括完成实名认证、提交招募申请、招募通过和首次任务执行；用于观察最新转化进度，不强制限定注册后 30 天。</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="52" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>按所选统计时间展示新增注册、活跃用户和 90 天未活跃用户变化；90 天未活跃用户为统计日首次达到连续 90 天无登录且无有效任务行为的去重用户数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="52" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>新用户转化漏斗</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>点击留存矩阵中的注册周期后，展示该批新用户截至所选统计期末到达各转化阶段的人数，包括完成实名认证、提交招募申请、招募通过和首次任务执行；用于观察最新转化进度，不强制限定注册后 30 天。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="52" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>新注册用户</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>所选注册周期内完成注册的去重用户数，是新用户转化漏斗和留存矩阵联动分析的基准用户数。</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="52" customHeight="1">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
+    <row r="29" ht="52" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>完成实名认证</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>所选注册周期用户中，截至当前已完成实名认证的去重用户数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="52" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>所选注册周期用户中，截至所选统计期末已完成实名认证的去重用户数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="52" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>提交招募申请</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>所选注册周期用户中，截至当前至少提交过一次招募申请的去重用户数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="52" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>所选注册周期用户中，截至所选统计期末至少提交过一次招募申请的去重用户数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="52" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>招募通过</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>所选注册周期用户中，截至当前至少有一个招募申请审核通过的去重用户数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="52" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>所选注册周期用户中，截至所选统计期末至少有一个招募申请审核通过的去重用户数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="52" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>首次任务执行</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>所选注册周期用户中，截至当前已产生首次有效任务行为的去重用户数；有效任务行为建议优先使用首次有效任务提交。</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="52" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>所选注册周期用户中，截至所选统计期末已产生首次有效任务行为的去重用户数；有效任务行为建议优先使用首次有效任务提交。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="52" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>环节转化率</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr">
         <is>
           <t>当前阶段达成人数/上一阶段达成人数；首个阶段按 100% 展示。</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="52" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
+    <row r="34" ht="52" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>累计转化率</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>当前阶段达成人数/该漏斗入组的新注册用户数。</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="52" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
+    <row r="35" ht="52" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>较上一步流失</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>上一阶段达成人数减去当前阶段达成人数，用于识别相邻阶段掉队规模。</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="52" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
+    <row r="36" ht="52" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>用户留存矩阵（按注册周）</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>按注册周期分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率；点击某一注册周期可同步查看该批新用户截至当前的转化漏斗。</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="52" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>按注册周期分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率；点击某一注册周期可同步查看该批新用户截至所选统计期末的转化漏斗。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="52" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>注册分组用户数</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>指定注册周期内完成注册的去重用户数，是留存矩阵 D1/D7/D14/D30 留存率的基准用户数。</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="52" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
+    <row r="38" ht="52" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>D1 留存</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>指定注册周期用户中注册后第 1 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="52" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
+    <row r="39" ht="52" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>D7 留存</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>指定注册周期用户中注册后第 7 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="52" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
+    <row r="40" ht="52" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>D14 留存</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>指定注册周期用户中注册后第 14 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="52" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
+    <row r="41" ht="52" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>D30 留存</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>指定注册周期用户中注册后第 30 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="52" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
+    <row r="42" ht="52" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>用户生命周期阶段分布</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>按用户截至统计日的最新生命周期状态归类的去重用户数；各阶段占比按该阶段用户数/注册总用户数计算。</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="52" customHeight="1">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>按用户截至所选统计期末的最新生命周期状态归类的去重用户数；各阶段占比按该阶段用户数/注册总用户数计算，各阶段互斥统计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="52" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>新注册</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>截至统计日注册未满 7 天，且尚未进入实名认证、招募申请或任务执行阶段的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="52" customHeight="1">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>截至所选统计期末注册未满 7 天，且尚未进入实名认证、招募申请或任务执行阶段的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="52" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>待实名认证</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>已完成注册但尚未完成实名认证，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="52" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
+    <row r="45" ht="52" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>未申请过招募</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>已完成实名认证但从未提交招募申请，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="52" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
+    <row r="46" ht="52" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>招募审核中</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>至少提交过一次招募申请，且最新有效申请仍处于待审核或审核中状态的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="52" customHeight="1">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
+    <row r="47" ht="52" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>招募申请通过</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>至少有一个招募申请已审核通过，但尚未产生有效任务执行行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="52" customHeight="1">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
+    <row r="48" ht="52" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>活跃执行中</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>近 30 天内有有效任务领取、进入任务、提交或质检相关行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="52" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
+    <row r="49" ht="52" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>30日未活跃</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>连续 30 天无登录且无有效任务行为，但尚未达到 60 天沉睡或 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="52" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
+    <row r="50" ht="52" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>60日沉睡</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>连续 60 天无登录且无有效任务行为，但尚未达到 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="52" customHeight="1">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
+    <row r="51" ht="52" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
         <is>
           <t>已流失用户</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>截至统计日连续 90 天无登录且无有效任务行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算，重新登录或产生有效任务行为后退出已流失状态。</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="52" customHeight="1">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>截至所选统计期末连续 90 天无登录且无有效任务行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算，重新登录或产生有效任务行为后退出已流失状态。</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="52" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>转化流失断点分析</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>按相邻转化环节展示进入该环节后未进入下一环节的流失人数和流失率，用于定位转化阻塞点；不等同于 90 天未活跃/已流失用户。</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="52" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>按相邻转化环节展示进入该环节后未进入下一环节的流失人数和流失率，用于定位转化阻塞点；不展示跨环节平均流失率，不等同于 90 天未活跃或已流失用户。</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="52" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>转化环节流失人数</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>用户转化漏斗中进入指定环节后未进入下一环节的去重用户数；与转化环节流失率使用同一批进入该环节的用户作为基准。</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="52" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
+    <row r="54" ht="52" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>转化环节流失率</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
-        <is>
-          <t>进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数；用于比较相邻转化断点，不应对多个环节简单平均，不等同于 90 天未活跃/已流失用户。</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="52" customHeight="1">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数；用于比较相邻转化断点，不应对多个环节简单平均，不等同于 90 天未活跃或已流失用户。</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="52" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>最大流失断点</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>转化流失断点分析中流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位当前最明显的转化阻塞点。</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="52" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>转化流失断点分析中流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位所选统计时间内最明显的转化阻塞点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="52" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>用户平均生命周期时长</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>观察用户从注册到流失或当前日期的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="52" customHeight="1">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>观察用户从注册到流失或所选统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="52" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
         <is>
           <t>平均生命周期</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>纳入样本用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到当前日期，已流失按连续 90 天无登录且无有效任务行为判定。</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="52" customHeight="1">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>纳入样本用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到所选统计期末，已流失按连续 90 天无登录且无有效任务行为判定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="52" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>注册→首单</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="52" customHeight="1">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>增长&amp;留存</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
+    <row r="59" ht="52" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>增长&amp;留存</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>生命周期时长分布</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到当前日期。</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="52" customHeight="1">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到所选统计期末。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="52" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B58" s="6" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>新增招募单</t>
         </is>
       </c>
-      <c r="C58" s="7" t="inlineStr">
-        <is>
-          <t>所选时间范围内新创建的招募单数量，按招募单 ID 去重。</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="52" customHeight="1">
-      <c r="A59" s="6" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内新创建的招募单数量，按招募单 ID 去重；招募分析不跟随其他模块的日期筛选。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="52" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B59" s="6" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>进行中招募单</t>
         </is>
       </c>
-      <c r="C59" s="7" t="inlineStr">
-        <is>
-          <t>截至统计日状态为招募中，且仍可接收用户申请的招募单数量，按招募单 ID 去重。</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="52" customHeight="1">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>统计日当前状态为招募中，且仍可接收用户申请的招募单数量，按招募单 ID 去重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="52" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B60" s="6" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>已完成招募单</t>
         </is>
       </c>
-      <c r="C60" s="7" t="inlineStr">
-        <is>
-          <t>所选时间范围内状态为已完成的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成。</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="52" customHeight="1">
-      <c r="A61" s="6" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内状态变更为已完成的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="52" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B61" s="6" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>目标招募总人数</t>
         </is>
       </c>
-      <c r="C61" s="7" t="inlineStr">
-        <is>
-          <t>所选招募单计划招募人数的合计，按招募单目标人数汇总。</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="52" customHeight="1">
-      <c r="A62" s="6" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，招募单计划招募人数的合计，按招募单目标人数汇总。</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="52" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B62" s="6" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>招募通过总人数</t>
         </is>
       </c>
-      <c r="C62" s="7" t="inlineStr">
-        <is>
-          <t>所选范围内招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；不等同于已到位人数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="52" customHeight="1">
-      <c r="A63" s="6" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，招募申请审核通过的去重用户数，同一用户在同一招募单只计一次。</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="52" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B63" s="6" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
         <is>
           <t>总缺口人数</t>
         </is>
       </c>
-      <c r="C63" s="7" t="inlineStr">
-        <is>
-          <t>目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="52" customHeight="1">
-      <c r="A64" s="6" t="inlineStr">
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="52" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B64" s="6" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>整体通过率</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
-        <is>
-          <t>审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="52" customHeight="1">
-      <c r="A65" s="6" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="52" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B65" s="6" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>招募转化趋势</t>
         </is>
       </c>
-      <c r="C65" s="7" t="inlineStr">
-        <is>
-          <t>按日期展示申请率和通过率趋势；申请率为提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数，通过率为审核通过的招募申请数/已完成审核的招募申请数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="52" customHeight="1">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>按日期展示申请率和通过率趋势；申请率为当前招募分析统计范围内提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数，通过率为审核通过的招募申请数/已完成审核的招募申请数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="52" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>申请率</t>
         </is>
       </c>
-      <c r="C66" s="7" t="inlineStr">
-        <is>
-          <t>提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="52" customHeight="1">
-      <c r="A67" s="6" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="52" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B67" s="6" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>通过率</t>
         </is>
       </c>
-      <c r="C67" s="7" t="inlineStr">
-        <is>
-          <t>审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="52" customHeight="1">
-      <c r="A68" s="6" t="inlineStr">
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="52" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B68" s="6" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>招募单数</t>
         </is>
       </c>
-      <c r="C68" s="7" t="inlineStr">
-        <is>
-          <t>所选范围内招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量。</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="52" customHeight="1">
-      <c r="A69" s="6" t="inlineStr">
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内的招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量。</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="52" customHeight="1">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B69" s="6" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>目标人数</t>
         </is>
       </c>
-      <c r="C69" s="7" t="inlineStr">
-        <is>
-          <t>所选招募单计划招募人数的合计，按招募单目标人数汇总。</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="52" customHeight="1">
-      <c r="A70" s="6" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，招募单计划招募人数的合计，按招募单目标人数汇总。</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="52" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B70" s="6" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>申请人数</t>
         </is>
       </c>
-      <c r="C70" s="7" t="inlineStr">
-        <is>
-          <t>所选范围内提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次。</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="52" customHeight="1">
-      <c r="A71" s="6" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="52" customHeight="1">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B71" s="6" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>招募通过人数</t>
         </is>
       </c>
-      <c r="C71" s="7" t="inlineStr">
-        <is>
-          <t>所选范围内招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；不等同于已到位人数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="52" customHeight="1">
-      <c r="A72" s="6" t="inlineStr">
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，招募申请审核通过的去重用户数，同一用户在同一招募单只计一次。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="52" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B72" s="6" t="inlineStr">
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>缺口人数</t>
         </is>
       </c>
-      <c r="C72" s="7" t="inlineStr">
-        <is>
-          <t>目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="52" customHeight="1">
-      <c r="A73" s="6" t="inlineStr">
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="52" customHeight="1">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B73" s="6" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>缺口率</t>
         </is>
       </c>
-      <c r="C73" s="7" t="inlineStr">
-        <is>
-          <t>缺口人数/目标招募人数；目标人数为 0 时不计算。</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="52" customHeight="1">
-      <c r="A74" s="6" t="inlineStr">
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，缺口人数/目标招募人数；目标人数为 0 时不计算。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="52" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B74" s="6" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>平均审核周期</t>
         </is>
       </c>
-      <c r="C74" s="7" t="inlineStr">
-        <is>
-          <t>已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="52" customHeight="1">
-      <c r="A75" s="6" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>当前招募分析统计范围内，已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="52" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B75" s="6" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>明细招募单状态</t>
         </is>
       </c>
-      <c r="C75" s="7" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>明细招募单当前状态，包含招募中、审核中、已暂停、已完成，用于配合招募单状态筛选查看不同状态下的招募表现。</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="52" customHeight="1">
-      <c r="A76" s="8" t="inlineStr">
+    <row r="78" ht="52" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B76" s="8" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>进行中任务数</t>
         </is>
       </c>
-      <c r="C76" s="9" t="inlineStr">
-        <is>
-          <t>截至统计日状态为进行中且可被执行或提交的任务数量，按任务 ID 去重。</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="52" customHeight="1">
-      <c r="A77" s="8" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>截至所选统计期末状态为进行中且可被执行或提交的任务数量，按任务 ID 去重。</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="52" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B77" s="8" t="inlineStr">
+      <c r="B79" s="2" t="inlineStr">
         <is>
           <t>参与人数</t>
         </is>
       </c>
-      <c r="C77" s="9" t="inlineStr">
-        <is>
-          <t>所选时间范围内产生领取、进入任务、提交或质检相关有效任务行为的去重用户数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="52" customHeight="1">
-      <c r="A78" s="8" t="inlineStr">
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内产生领取、进入任务、提交或质检相关有效任务行为的去重用户数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="52" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B78" s="8" t="inlineStr">
-        <is>
-          <t>总提交量</t>
-        </is>
-      </c>
-      <c r="C78" s="9" t="inlineStr">
-        <is>
-          <t>所选时间范围内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="52" customHeight="1">
-      <c r="A79" s="8" t="inlineStr">
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>提交量</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="52" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B79" s="8" t="inlineStr">
+      <c r="B81" s="2" t="inlineStr">
         <is>
           <t>标注质检通过率</t>
         </is>
       </c>
-      <c r="C79" s="9" t="inlineStr">
-        <is>
-          <t>标注任务中质检通过的数据条数/标注任务中已完成质检的数据条数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="52" customHeight="1">
-      <c r="A80" s="8" t="inlineStr">
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内，标注任务中质检通过的数据条数/标注任务中已完成质检的数据条数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="52" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B80" s="8" t="inlineStr">
-        <is>
-          <t>今日提交量</t>
-        </is>
-      </c>
-      <c r="C80" s="9" t="inlineStr">
-        <is>
-          <t>统计日内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="52" customHeight="1">
-      <c r="A81" s="8" t="inlineStr">
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>返工率</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内，被退回或要求返修的数据条数/已质检或已提交的数据条数，按业务选择同一口径。</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="52" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B81" s="8" t="inlineStr">
+      <c r="B83" s="2" t="inlineStr">
         <is>
           <t>人均日产能</t>
         </is>
       </c>
-      <c r="C81" s="9" t="inlineStr">
-        <is>
-          <t>统计日任务提交数据条数/统计日有有效任务行为的去重用户数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="52" customHeight="1">
-      <c r="A82" s="8" t="inlineStr">
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>所选统计日期的任务提交数据条数/同一统计日期有有效任务行为的去重用户数；选择周、月或近 N 天时建议展示区间日均。</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="52" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B82" s="8" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>采集质检通过率</t>
         </is>
       </c>
-      <c r="C82" s="9" t="inlineStr">
-        <is>
-          <t>采集任务中质检通过的数据条数/采集任务中已完成质检的数据条数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="52" customHeight="1">
-      <c r="A83" s="8" t="inlineStr">
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内，采集任务中质检通过的数据条数/采集任务中已完成质检的数据条数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="52" customHeight="1">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B83" s="8" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>数据产出趋势</t>
         </is>
       </c>
-      <c r="C83" s="9" t="inlineStr">
+      <c r="C85" s="3" t="inlineStr">
         <is>
           <t>按日期展示标注提交数据条数和采集提交数据条数，用于观察不同任务类型的数据产出变化。</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="52" customHeight="1">
-      <c r="A84" s="8" t="inlineStr">
+    <row r="86" ht="52" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B84" s="8" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>标注提交数据条数</t>
         </is>
       </c>
-      <c r="C84" s="9" t="inlineStr">
-        <is>
-          <t>所选时间范围内标注任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="52" customHeight="1">
-      <c r="A85" s="8" t="inlineStr">
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内标注任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="52" customHeight="1">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B85" s="8" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>采集提交数据条数</t>
         </is>
       </c>
-      <c r="C85" s="9" t="inlineStr">
-        <is>
-          <t>所选时间范围内采集任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="52" customHeight="1">
-      <c r="A86" s="8" t="inlineStr">
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>所选统计时间内采集任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="52" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B86" s="8" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>后续质检通过率趋势</t>
         </is>
       </c>
-      <c r="C86" s="9" t="inlineStr">
+      <c r="C88" s="3" t="inlineStr">
         <is>
           <t>按日期展示后续质检通过率；后续质检通过率为首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数，不拆分具体轮次。</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="52" customHeight="1">
-      <c r="A87" s="8" t="inlineStr">
+    <row r="89" ht="52" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B87" s="8" t="inlineStr">
+      <c r="B89" s="2" t="inlineStr">
         <is>
           <t>后续质检通过率</t>
         </is>
       </c>
-      <c r="C87" s="9" t="inlineStr">
+      <c r="C89" s="3" t="inlineStr">
         <is>
           <t>首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数；不拆分具体轮次。</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="52" customHeight="1">
-      <c r="A88" s="8" t="inlineStr">
+    <row r="90" ht="15" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B88" s="8" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>错误类型分布</t>
         </is>
       </c>
-      <c r="C88" s="9" t="inlineStr">
+      <c r="C90" s="3" t="inlineStr">
         <is>
           <t>按错误类型展示质检错误结构，错误类型占比为指定错误类型的错误条数/全部质检错误条数。</t>
         </is>
       </c>
     </row>
-    <row r="89" ht="52" customHeight="1">
-      <c r="A89" s="8" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B89" s="8" t="inlineStr">
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>错误类型占比</t>
         </is>
       </c>
-      <c r="C89" s="9" t="inlineStr">
+      <c r="C91" s="3" t="inlineStr">
         <is>
           <t>指定错误类型的错误条数/全部质检错误条数，用于观察错误结构。</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="8" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
         <is>
           <t>任务&amp;质量</t>
         </is>
       </c>
-      <c r="B90" s="8" t="inlineStr">
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>新用户错误占比</t>
         </is>
       </c>
-      <c r="C90" s="9" t="inlineStr">
+      <c r="C92" s="3" t="inlineStr">
         <is>
           <t>新用户产生的质检错误条数/全部质检错误条数；新用户口径需按平台注册或首单时间窗统一定义。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C89"/>
+  <autoFilter ref="A1:C92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;L&amp;"Calibri"&amp;10 &amp;K000000_x000d_# This content is for internal use only</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify metric time scopes
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -814,7 +814,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>截至所选统计期末，平台累计完成注册的去重众包用户数，以用户 ID 去重。</t>
+          <t>截至核心指标时间期末，平台累计完成注册的去重众包用户数，以用户 ID 去重。</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>所选统计时间内完成注册的去重用户数，以用户 ID 去重；选择日时展示单日数据，选择周、月或近 N 天时展示区间汇总数据。</t>
+          <t>核心指标时间内完成注册的去重用户数，以用户 ID 去重；选择日时展示单日数据，选择周、月或近 N 天时展示区间汇总数据。</t>
         </is>
       </c>
     </row>
@@ -843,12 +843,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>DAU 活跃</t>
+          <t>活跃用户</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>所选统计日期内至少发生一次登录、访问核心页面或有效任务行为的去重用户数；选择周、月或近 N 天时可按区间口径汇总展示。</t>
+          <t>核心指标时间内至少发生一次登录、访问核心页面或有效任务行为的去重用户数；选择日时为单日活跃用户，选择周、月或近 N 天时为区间活跃用户。</t>
         </is>
       </c>
     </row>
@@ -860,12 +860,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>MAU 月活用户</t>
+          <t>近30天活跃用户</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>近 30 天或自然月内至少发生一次登录、访问核心页面或有效任务行为的去重用户数。</t>
+          <t>截至核心指标时间期末，近 30 天内至少发生一次登录、访问核心页面或有效任务行为的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -877,12 +877,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>平台月活跃用户占比</t>
+          <t>活跃用户占比</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>近 30 天或自然月活跃用户数/截至所选统计期末的注册总用户数。</t>
+          <t>截至核心指标时间期末的近 30 天活跃用户数/截至同一统计期末的注册总用户数。</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>所选统计时间内完成注册的新访客数/同一统计时间内首次访问平台的新访客数。</t>
+          <t>核心指标时间内完成注册的新访客数/同一统计时间内首次访问平台的新访客数。</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>已完成实名认证的注册用户数/具备实名认证资格的注册用户数；未开始认证和认证失败均不计入已认证用户数。</t>
+          <t>核心指标时间内注册且截至统计期末已完成实名认证的用户数/核心指标时间内具备实名认证资格的注册用户数；时间筛选的是用户注册时间，未开始认证和认证失败均不计入已认证用户数。</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>完成实名认证后提交过至少一次招募申请的用户数/完成实名认证且可申请招募的用户数。</t>
+          <t>核心指标时间内注册且截至统计期末完成实名认证后提交过至少一次招募申请的用户数/核心指标时间内完成实名认证且可申请招募的用户数；时间筛选的是用户注册时间。</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>按所选统计时间展示新增注册、活跃用户和 90 天未活跃用户变化；90 天未活跃用户为统计日首次达到连续 90 天无登录且无有效任务行为的去重用户数。</t>
+          <t>使用独立的趋势时间筛选，筛选的是事件发生时间；按该时间展示新增注册、活跃用户和首次达到 90 天未活跃用户变化。</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>点击留存矩阵中的注册周期后，展示该批新用户截至所选统计期末到达各转化阶段的人数，包括完成实名认证、提交招募申请、招募通过和首次任务执行；用于观察最新转化进度，不强制限定注册后 30 天。</t>
+          <t>与用户留存矩阵联动，筛选的是用户注册时间；点击留存矩阵中的注册周期后，展示该批新用户截至统计期末到达完成实名认证、提交招募申请、招募通过和首次任务执行等阶段的人数。</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>所选注册周期内完成注册的去重用户数，是新用户转化漏斗和留存矩阵联动分析的基准用户数。</t>
+          <t>所选注册时间内完成注册的去重用户数，是新用户转化漏斗和留存矩阵联动分析的基准用户数。</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>所选注册周期用户中，截至所选统计期末已完成实名认证的去重用户数。</t>
+          <t>所选注册时间内入组的用户中，截至统计期末已完成实名认证的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>所选注册周期用户中，截至所选统计期末至少提交过一次招募申请的去重用户数。</t>
+          <t>所选注册时间内入组的用户中，截至统计期末至少提交过一次招募申请的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>所选注册周期用户中，截至所选统计期末至少有一个招募申请审核通过的去重用户数。</t>
+          <t>所选注册时间内入组的用户中，截至统计期末至少有一个招募申请审核通过的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>所选注册周期用户中，截至所选统计期末已产生首次有效任务行为的去重用户数；有效任务行为建议优先使用首次有效任务提交。</t>
+          <t>所选注册时间内入组的用户中，截至统计期末已产生首次有效任务行为的去重用户数；有效任务行为建议优先使用首次有效任务提交。</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>按注册周期分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率；点击某一注册周期可同步查看该批新用户截至所选统计期末的转化漏斗。</t>
+          <t>使用独立的注册时间筛选，按注册周期分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率；点击某一注册周期可同步查看该批新用户的当前转化漏斗。</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>指定注册周期内完成注册的去重用户数，是留存矩阵 D1/D7/D14/D30 留存率的基准用户数。</t>
+          <t>所选注册时间内完成注册的去重用户数，是留存矩阵 D1/D7/D14/D30 留存率的基准用户数。</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>按用户截至所选统计期末的最新生命周期状态归类的去重用户数；各阶段占比按该阶段用户数/注册总用户数计算，各阶段互斥统计。</t>
+          <t>使用独立的快照时间筛选，按快照时点用户最新生命周期状态归类的去重用户数；各阶段占比按该阶段用户数/注册总用户数计算，各阶段互斥统计。</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>截至所选统计期末注册未满 7 天，且尚未进入实名认证、招募申请或任务执行阶段的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至快照时间注册未满 7 天，且尚未进入实名认证、招募申请或任务执行阶段的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>已完成注册但尚未完成实名认证，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至快照时间已完成注册但尚未完成实名认证，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>已完成实名认证但从未提交招募申请，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至快照时间已完成实名认证但从未提交招募申请，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1290,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>至少提交过一次招募申请，且最新有效申请仍处于待审核或审核中状态的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至快照时间至少提交过一次招募申请，且最新有效申请仍处于待审核或审核中状态的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>至少有一个招募申请已审核通过，但尚未产生有效任务执行行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至快照时间至少有一个招募申请已审核通过，但尚未产生有效任务执行行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>近 30 天内有有效任务领取、进入任务、提交或质检相关行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至快照时间近 30 天内有有效任务领取、进入任务、提交或质检相关行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>连续 30 天无登录且无有效任务行为，但尚未达到 60 天沉睡或 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至快照时间连续 30 天无登录且无有效任务行为，但尚未达到 60 天沉睡或 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>连续 60 天无登录且无有效任务行为，但尚未达到 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至快照时间连续 60 天无登录且无有效任务行为，但尚未达到 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>截至所选统计期末连续 90 天无登录且无有效任务行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算，重新登录或产生有效任务行为后退出已流失状态。</t>
+          <t>截至快照时间连续 90 天无登录且无有效任务行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算，重新登录或产生有效任务行为后退出已流失状态。</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>按相邻转化环节展示进入该环节后未进入下一环节的流失人数和流失率，用于定位转化阻塞点；不展示跨环节平均流失率，不等同于 90 天未活跃或已流失用户。</t>
+          <t>使用独立的入组注册时间筛选，观察该批用户截至统计期末在相邻转化环节的流失人数和流失率；不展示跨环节平均流失率，不等同于 90 天未活跃或已流失用户。</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>用户转化漏斗中进入指定环节后未进入下一环节的去重用户数；与转化环节流失率使用同一批进入该环节的用户作为基准。</t>
+          <t>所选入组注册时间内用户在进入指定环节后未进入下一环节的去重用户数；与转化环节流失率使用同一批进入该环节的用户作为基准。</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>转化流失断点分析中流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位所选统计时间内最明显的转化阻塞点。</t>
+          <t>转化流失断点分析中流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位所选入组注册时间内最明显的转化阻塞点。</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>观察用户从注册到流失或所选统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
+          <t>使用独立的注册时间筛选，观察该批用户从注册到流失判定或统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1477,7 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>纳入样本用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到所选统计期末，已流失按连续 90 天无登录且无有效任务行为判定。</t>
+          <t>所选注册时间内入组用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到统计期末，已流失按连续 90 天无登录且无有效任务行为判定。</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
+          <t>所选注册时间内入组用户从完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到所选统计期末。</t>
+          <t>所选注册时间内入组用户的生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到统计期末。</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内新创建的招募单数量，按招募单 ID 去重；招募分析不跟随其他模块的日期筛选。</t>
+          <t>统计日新创建，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；统计日为 T+1 最新可用日期，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1545,7 +1545,7 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>统计日当前状态为招募中，且仍可接收用户申请的招募单数量，按招募单 ID 去重。</t>
+          <t>统计日当前状态为招募中、仍可接收用户申请，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内状态变更为已完成的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成。</t>
+          <t>统计日状态变更为已完成，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，招募单计划招募人数的合计，按招募单目标人数汇总。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，招募申请审核通过的去重用户数，同一用户在同一招募单只计一次。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>按日期展示申请率和通过率趋势；申请率为当前招募分析统计范围内提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数，通过率为审核通过的招募申请数/已完成审核的招募申请数。</t>
+          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示申请率和通过率趋势。</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，提交招募申请的去重用户数/访问或曝光该招募单且具备申请资格的去重用户数。</t>
+          <t>所选趋势时间内，符合当前领域筛选的提交招募申请去重用户数/访问或曝光该招募单且具备申请资格的去重用户数；招募指标卡片默认按统计日与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，审核通过的招募申请数/已完成审核的招募申请数；待审核申请不纳入计算。</t>
+          <t>所选趋势时间内，符合当前领域筛选的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，招募指标卡片默认按统计日与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内的招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，招募单计划招募人数的合计，按招募单目标人数汇总。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，招募申请审核通过的去重用户数，同一用户在同一招募单只计一次。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，缺口人数/目标招募人数；目标人数为 0 时不计算。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的缺口人数/目标招募人数；目标人数为 0 时不计算，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>当前招募分析统计范围内，已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围、已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>明细招募单当前状态，包含招募中、审核中、已暂停、已完成，用于配合招募单状态筛选查看不同状态下的招募表现。</t>
+          <t>明细招募单在统计日的当前状态，包含招募中、审核中、已暂停、已完成，用于配合招募单状态筛选查看不同状态下的招募表现。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Simplify growth retention filters
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -831,7 +831,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>核心指标时间内完成注册的去重用户数，以用户 ID 去重；选择日时展示单日数据，选择周、月或近 N 天时展示区间汇总数据。</t>
+          <t>核心指标时间内完成注册的去重用户数，以用户 ID 去重；时间筛选的是用户注册成功时间。</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>核心指标时间内至少发生一次登录、访问核心页面或有效任务行为的去重用户数；选择日时为单日活跃用户，选择周、月或近 N 天时为区间活跃用户。</t>
+          <t>核心指标时间内至少发生一次登录、访问核心页面或有效任务行为的去重用户数；时间筛选的是活跃事件发生时间，选择日时为单日活跃用户，选择周、月或近 N 天时为区间活跃用户。</t>
         </is>
       </c>
     </row>
@@ -860,12 +860,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>近30天活跃用户</t>
+          <t>活跃用户占比</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>截至核心指标时间期末，近 30 天内至少发生一次登录、访问核心页面或有效任务行为的去重用户数。</t>
+          <t>截至核心指标时间期末的近 30 天活跃用户数/截至同一统计期末的注册总用户数。</t>
         </is>
       </c>
     </row>
@@ -877,12 +877,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>活跃用户占比</t>
+          <t>新访客注册转化率</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>截至核心指标时间期末的近 30 天活跃用户数/截至同一统计期末的注册总用户数。</t>
+          <t>核心指标时间内首次访问平台的新访客中，截至该统计期末完成注册的新访客数/同一核心指标时间内首次访问平台的新访客数；时间筛选的是新访客首次访问时间。</t>
         </is>
       </c>
     </row>
@@ -894,12 +894,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>新访客注册转化率</t>
+          <t>实名认证率</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>核心指标时间内完成注册的新访客数/同一统计时间内首次访问平台的新访客数。</t>
+          <t>核心指标时间内注册且截至该统计期末已完成实名认证的用户数/同一核心指标时间内具备实名认证资格的注册用户数；时间筛选的是用户注册时间，未开始认证和认证失败均不计入已认证用户数。</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>实名认证率</t>
+          <t>招募申请率</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>核心指标时间内注册且截至统计期末已完成实名认证的用户数/核心指标时间内具备实名认证资格的注册用户数；时间筛选的是用户注册时间，未开始认证和认证失败均不计入已认证用户数。</t>
+          <t>核心指标时间内注册且截至该统计期末完成实名认证后提交过至少一次招募申请的用户数/同一核心指标时间内完成实名认证且可申请招募的用户数；时间筛选的是用户注册时间。</t>
         </is>
       </c>
     </row>
@@ -928,12 +928,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>招募申请率</t>
+          <t>用户增长趋势</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>核心指标时间内注册且截至统计期末完成实名认证后提交过至少一次招募申请的用户数/核心指标时间内完成实名认证且可申请招募的用户数；时间筛选的是用户注册时间。</t>
+          <t>固定展示近 7 日趋势，时间口径为事件发生日；每日展示新增注册、活跃用户和首次达到 90 天未活跃的用户变化。</t>
         </is>
       </c>
     </row>
@@ -945,12 +945,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>用户增长趋势</t>
+          <t>新用户转化漏斗</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>使用独立的趋势时间筛选，筛选的是事件发生时间；按该时间展示新增注册、活跃用户和首次达到 90 天未活跃用户变化。</t>
+          <t>与用户留存矩阵联动，时间口径为留存矩阵中选定的注册周；展示该批新用户截至 T+1 最新统计日到达完成实名认证、提交招募申请、招募通过和首次任务执行等阶段的人数。</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>新用户转化漏斗</t>
+          <t>新注册用户</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>与用户留存矩阵联动，筛选的是用户注册时间；点击留存矩阵中的注册周期后，展示该批新用户截至统计期末到达完成实名认证、提交招募申请、招募通过和首次任务执行等阶段的人数。</t>
+          <t>留存矩阵中选定注册周内完成注册的去重用户数，是新用户转化漏斗和留存矩阵联动分析的基准用户数。</t>
         </is>
       </c>
     </row>
@@ -979,12 +979,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>新注册用户</t>
+          <t>完成实名认证</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>所选注册时间内完成注册的去重用户数，是新用户转化漏斗和留存矩阵联动分析的基准用户数。</t>
+          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日已完成实名认证的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -996,12 +996,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>完成实名认证</t>
+          <t>提交招募申请</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>所选注册时间内入组的用户中，截至统计期末已完成实名认证的去重用户数。</t>
+          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日至少提交过一次招募申请的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1013,12 +1013,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>提交招募申请</t>
+          <t>招募通过</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>所选注册时间内入组的用户中，截至统计期末至少提交过一次招募申请的去重用户数。</t>
+          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日至少有一个招募申请审核通过的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1030,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>招募通过</t>
+          <t>首次任务执行</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>所选注册时间内入组的用户中，截至统计期末至少有一个招募申请审核通过的去重用户数。</t>
+          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日已产生首次有效任务行为的去重用户数；有效任务行为建议优先使用首次有效任务提交。</t>
         </is>
       </c>
     </row>
@@ -1047,12 +1047,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>首次任务执行</t>
+          <t>环节转化率</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>所选注册时间内入组的用户中，截至统计期末已产生首次有效任务行为的去重用户数；有效任务行为建议优先使用首次有效任务提交。</t>
+          <t>当前阶段达成人数/上一阶段达成人数；首个阶段按 100% 展示。</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>环节转化率</t>
+          <t>累计转化率</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>当前阶段达成人数/上一阶段达成人数；首个阶段按 100% 展示。</t>
+          <t>当前阶段达成人数/该漏斗入组的新注册用户数。</t>
         </is>
       </c>
     </row>
@@ -1081,12 +1081,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>累计转化率</t>
+          <t>较上一步流失</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>当前阶段达成人数/该漏斗入组的新注册用户数。</t>
+          <t>上一阶段达成人数减去当前阶段达成人数，用于识别相邻阶段掉队规模。</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>较上一步流失</t>
+          <t>用户留存矩阵（按注册周）</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>上一阶段达成人数减去当前阶段达成人数，用于识别相邻阶段掉队规模。</t>
+          <t>只提供周数筛选，用于选择近 N 个注册周；按注册周分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率，点击某一注册周可同步查看该批新用户的当前转化漏斗。</t>
         </is>
       </c>
     </row>
@@ -1115,12 +1115,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>用户留存矩阵（按注册周）</t>
+          <t>注册分组用户数</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>使用独立的注册时间筛选，按注册周期分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率；点击某一注册周期可同步查看该批新用户的当前转化漏斗。</t>
+          <t>留存矩阵按近 N 个注册周筛选，指定注册周内完成注册的去重用户数，是 D1/D7/D14/D30 留存率的基准用户数。</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1132,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>注册分组用户数</t>
+          <t>D1 留存</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>所选注册时间内完成注册的去重用户数，是留存矩阵 D1/D7/D14/D30 留存率的基准用户数。</t>
+          <t>指定注册周期用户中注册后第 1 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
@@ -1149,12 +1149,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>D1 留存</t>
+          <t>D7 留存</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>指定注册周期用户中注册后第 1 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
+          <t>指定注册周期用户中注册后第 7 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>D7 留存</t>
+          <t>D14 留存</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>指定注册周期用户中注册后第 7 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
+          <t>指定注册周期用户中注册后第 14 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
@@ -1183,12 +1183,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>D14 留存</t>
+          <t>D30 留存</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>指定注册周期用户中注册后第 14 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
+          <t>指定注册周期用户中注册后第 30 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
@@ -1200,12 +1200,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>D30 留存</t>
+          <t>用户生命周期阶段分布</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>指定注册周期用户中注册后第 30 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
+          <t>不提供时间筛选，按 T+1 最新统计日快照统计用户最新生命周期状态；各阶段占比按该阶段用户数/注册总用户数计算，各阶段互斥统计。</t>
         </is>
       </c>
     </row>
@@ -1217,12 +1217,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>用户生命周期阶段分布</t>
+          <t>新注册</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>使用独立的快照时间筛选，按快照时点用户最新生命周期状态归类的去重用户数；各阶段占比按该阶段用户数/注册总用户数计算，各阶段互斥统计。</t>
+          <t>截至 T+1 最新统计日注册未满 7 天，且尚未进入实名认证、招募申请或任务执行阶段的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>新注册</t>
+          <t>待实名认证</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>截至快照时间注册未满 7 天，且尚未进入实名认证、招募申请或任务执行阶段的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日已完成注册但尚未完成实名认证，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1251,12 +1251,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>待实名认证</t>
+          <t>未申请过招募</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>截至快照时间已完成注册但尚未完成实名认证，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日已完成实名认证但从未提交招募申请，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1268,12 +1268,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>未申请过招募</t>
+          <t>招募审核中</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>截至快照时间已完成实名认证但从未提交招募申请，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日至少提交过一次招募申请，且最新有效申请仍处于待审核或审核中状态的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1285,12 +1285,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>招募审核中</t>
+          <t>招募申请通过</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>截至快照时间至少提交过一次招募申请，且最新有效申请仍处于待审核或审核中状态的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日至少有一个招募申请已审核通过，但尚未产生有效任务执行行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1302,12 +1302,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>招募申请通过</t>
+          <t>活跃执行中</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>截至快照时间至少有一个招募申请已审核通过，但尚未产生有效任务执行行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日近 30 天内有有效任务领取、进入任务、提交或质检相关行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>活跃执行中</t>
+          <t>30日未活跃</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>截至快照时间近 30 天内有有效任务领取、进入任务、提交或质检相关行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日连续 30 天无登录且无有效任务行为，但尚未达到 60 天沉睡或 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1336,12 +1336,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>30日未活跃</t>
+          <t>60日沉睡</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>截至快照时间连续 30 天无登录且无有效任务行为，但尚未达到 60 天沉睡或 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日连续 60 天无登录且无有效任务行为，但尚未达到 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1353,12 +1353,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>60日沉睡</t>
+          <t>已流失用户</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>截至快照时间连续 60 天无登录且无有效任务行为，但尚未达到 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日连续 90 天无登录且无有效任务行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算，重新登录或产生有效任务行为后退出已流失状态。</t>
         </is>
       </c>
     </row>
@@ -1370,12 +1370,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>已流失用户</t>
+          <t>转化流失断点分析</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>截至快照时间连续 90 天无登录且无有效任务行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算，重新登录或产生有效任务行为后退出已流失状态。</t>
+          <t>暂不提供筛选，按当前样本截至 T+1 最新统计日观察相邻转化环节的流失人数和流失率；不展示跨环节平均流失率，不等同于 90 天未活跃或已流失用户。</t>
         </is>
       </c>
     </row>
@@ -1387,12 +1387,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>转化流失断点分析</t>
+          <t>转化环节流失人数</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>使用独立的入组注册时间筛选，观察该批用户截至统计期末在相邻转化环节的流失人数和流失率；不展示跨环节平均流失率，不等同于 90 天未活跃或已流失用户。</t>
+          <t>当前样本用户截至 T+1 最新统计日进入指定环节后未进入下一环节的去重用户数；与转化环节流失率使用同一批进入该环节的用户作为基准。</t>
         </is>
       </c>
     </row>
@@ -1404,12 +1404,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>转化环节流失人数</t>
+          <t>转化环节流失率</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>所选入组注册时间内用户在进入指定环节后未进入下一环节的去重用户数；与转化环节流失率使用同一批进入该环节的用户作为基准。</t>
+          <t>当前样本用户截至 T+1 最新统计日进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数；用于比较相邻转化断点，不应对多个环节简单平均，不等同于 90 天未活跃或已流失用户。</t>
         </is>
       </c>
     </row>
@@ -1421,12 +1421,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>转化环节流失率</t>
+          <t>最大流失断点</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数；用于比较相邻转化断点，不应对多个环节简单平均，不等同于 90 天未活跃或已流失用户。</t>
+          <t>当前样本用户截至 T+1 最新统计日流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位最明显的转化阻塞点。</t>
         </is>
       </c>
     </row>
@@ -1438,12 +1438,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>最大流失断点</t>
+          <t>用户平均生命周期时长</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>转化流失断点分析中流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位所选入组注册时间内最明显的转化阻塞点。</t>
+          <t>暂不提供筛选，按当前样本截至 T+1 最新统计日观察用户从注册到流失判定或统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
         </is>
       </c>
     </row>
@@ -1455,12 +1455,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>用户平均生命周期时长</t>
+          <t>平均生命周期</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>使用独立的注册时间筛选，观察该批用户从注册到流失判定或统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
+          <t>当前样本用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到 T+1 最新统计日，已流失按连续 90 天无登录且无有效任务行为判定。</t>
         </is>
       </c>
     </row>
@@ -1472,12 +1472,12 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>平均生命周期</t>
+          <t>注册→首单</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>所选注册时间内入组用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到统计期末，已流失按连续 90 天无登录且无有效任务行为判定。</t>
+          <t>当前样本用户从完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
         </is>
       </c>
     </row>
@@ -1489,29 +1489,29 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>注册→首单</t>
+          <t>生命周期时长分布</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>所选注册时间内入组用户从完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
+          <t>生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到 T+1 最新统计日。</t>
         </is>
       </c>
     </row>
     <row r="59" ht="52" customHeight="1">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>增长&amp;留存</t>
+          <t>招募分析</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>生命周期时长分布</t>
+          <t>新增招募单</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>所选注册时间内入组用户的生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到统计期末。</t>
+          <t>统计日新创建，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；统计日为 T+1 最新可用日期，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1523,12 +1523,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>新增招募单</t>
+          <t>进行中招募单</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>统计日新创建，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；统计日为 T+1 最新可用日期，默认与前一统计日对比。</t>
+          <t>统计日当前状态为招募中、仍可接收用户申请，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1540,12 +1540,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>进行中招募单</t>
+          <t>已完成招募单</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>统计日当前状态为招募中、仍可接收用户申请，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；默认与前一统计日对比。</t>
+          <t>统计日状态变更为已完成，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1557,12 +1557,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>已完成招募单</t>
+          <t>目标招募总人数</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>统计日状态变更为已完成，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成，默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>目标招募总人数</t>
+          <t>招募通过总人数</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1591,12 +1591,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>招募通过总人数</t>
+          <t>总缺口人数</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1608,12 +1608,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>总缺口人数</t>
+          <t>整体通过率</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1625,12 +1625,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>整体通过率</t>
+          <t>招募转化趋势</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，默认与前一统计日对比。</t>
+          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示申请率和通过率趋势。</t>
         </is>
       </c>
     </row>
@@ -1642,12 +1642,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>招募转化趋势</t>
+          <t>申请率</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示申请率和通过率趋势。</t>
+          <t>所选趋势时间内，符合当前领域筛选的提交招募申请去重用户数/访问或曝光该招募单且具备申请资格的去重用户数；招募指标卡片默认按统计日与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1659,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>申请率</t>
+          <t>通过率</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>所选趋势时间内，符合当前领域筛选的提交招募申请去重用户数/访问或曝光该招募单且具备申请资格的去重用户数；招募指标卡片默认按统计日与前一统计日对比。</t>
+          <t>所选趋势时间内，符合当前领域筛选的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，招募指标卡片默认按统计日与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1676,12 +1676,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>通过率</t>
+          <t>招募单数</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>所选趋势时间内，符合当前领域筛选的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，招募指标卡片默认按统计日与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1693,12 +1693,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>招募单数</t>
+          <t>目标人数</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量，默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1710,12 +1710,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>目标人数</t>
+          <t>申请人数</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1727,12 +1727,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>申请人数</t>
+          <t>招募通过人数</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次；默认与前一统计日对比。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1744,12 +1744,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>招募通过人数</t>
+          <t>缺口人数</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1761,12 +1761,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>缺口人数</t>
+          <t>缺口率</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的缺口人数/目标招募人数；目标人数为 0 时不计算，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1778,12 +1778,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>缺口率</t>
+          <t>平均审核周期</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的缺口人数/目标招募人数；目标人数为 0 时不计算，默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围、已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1795,29 +1795,29 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>平均审核周期</t>
+          <t>明细招募单状态</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围、已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计；默认与前一统计日对比。</t>
+          <t>明细招募单在统计日的当前状态，包含招募中、审核中、已暂停、已完成，用于配合招募单状态筛选查看不同状态下的招募表现。</t>
         </is>
       </c>
     </row>
     <row r="77" ht="52" customHeight="1">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>招募分析</t>
+          <t>任务&amp;质量</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>明细招募单状态</t>
+          <t>进行中任务数</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>明细招募单在统计日的当前状态，包含招募中、审核中、已暂停、已完成，用于配合招募单状态筛选查看不同状态下的招募表现。</t>
+          <t>截至所选统计期末状态为进行中且可被执行或提交的任务数量，按任务 ID 去重。</t>
         </is>
       </c>
     </row>
@@ -1829,12 +1829,12 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>进行中任务数</t>
+          <t>参与人数</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>截至所选统计期末状态为进行中且可被执行或提交的任务数量，按任务 ID 去重。</t>
+          <t>所选统计时间内产生领取、进入任务、提交或质检相关有效任务行为的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1846,12 +1846,12 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>参与人数</t>
+          <t>提交量</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
-          <t>所选统计时间内产生领取、进入任务、提交或质检相关有效任务行为的去重用户数。</t>
+          <t>所选统计时间内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
         </is>
       </c>
     </row>
@@ -1863,12 +1863,12 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>提交量</t>
+          <t>标注质检通过率</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>所选统计时间内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
+          <t>所选统计时间内，标注任务中质检通过的数据条数/标注任务中已完成质检的数据条数。</t>
         </is>
       </c>
     </row>
@@ -1880,12 +1880,12 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>标注质检通过率</t>
+          <t>返工率</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>所选统计时间内，标注任务中质检通过的数据条数/标注任务中已完成质检的数据条数。</t>
+          <t>所选统计时间内，被退回或要求返修的数据条数/已质检或已提交的数据条数，按业务选择同一口径。</t>
         </is>
       </c>
     </row>
@@ -1897,12 +1897,12 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>返工率</t>
+          <t>人均日产能</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>所选统计时间内，被退回或要求返修的数据条数/已质检或已提交的数据条数，按业务选择同一口径。</t>
+          <t>所选统计日期的任务提交数据条数/同一统计日期有有效任务行为的去重用户数；选择周、月或近 N 天时建议展示区间日均。</t>
         </is>
       </c>
     </row>
@@ -1914,12 +1914,12 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>人均日产能</t>
+          <t>采集质检通过率</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>所选统计日期的任务提交数据条数/同一统计日期有有效任务行为的去重用户数；选择周、月或近 N 天时建议展示区间日均。</t>
+          <t>所选统计时间内，采集任务中质检通过的数据条数/采集任务中已完成质检的数据条数。</t>
         </is>
       </c>
     </row>
@@ -1931,12 +1931,12 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>采集质检通过率</t>
+          <t>数据产出趋势</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>所选统计时间内，采集任务中质检通过的数据条数/采集任务中已完成质检的数据条数。</t>
+          <t>按日期展示标注提交数据条数和采集提交数据条数，用于观察不同任务类型的数据产出变化。</t>
         </is>
       </c>
     </row>
@@ -1948,12 +1948,12 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>数据产出趋势</t>
+          <t>标注提交数据条数</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>按日期展示标注提交数据条数和采集提交数据条数，用于观察不同任务类型的数据产出变化。</t>
+          <t>所选统计时间内标注任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
         </is>
       </c>
     </row>
@@ -1965,12 +1965,12 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>标注提交数据条数</t>
+          <t>采集提交数据条数</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
         <is>
-          <t>所选统计时间内标注任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
+          <t>所选统计时间内采集任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
         </is>
       </c>
     </row>
@@ -1982,12 +1982,12 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>采集提交数据条数</t>
+          <t>后续质检通过率趋势</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>所选统计时间内采集任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
+          <t>按日期展示后续质检通过率；后续质检通过率为首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数，不拆分具体轮次。</t>
         </is>
       </c>
     </row>
@@ -1999,12 +1999,12 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>后续质检通过率趋势</t>
+          <t>后续质检通过率</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
         <is>
-          <t>按日期展示后续质检通过率；后续质检通过率为首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数，不拆分具体轮次。</t>
+          <t>首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数；不拆分具体轮次。</t>
         </is>
       </c>
     </row>
@@ -2016,12 +2016,12 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>后续质检通过率</t>
+          <t>错误类型分布</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数；不拆分具体轮次。</t>
+          <t>按错误类型展示质检错误结构，错误类型占比为指定错误类型的错误条数/全部质检错误条数。</t>
         </is>
       </c>
     </row>
@@ -2033,12 +2033,12 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>错误类型分布</t>
+          <t>错误类型占比</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>按错误类型展示质检错误结构，错误类型占比为指定错误类型的错误条数/全部质检错误条数。</t>
+          <t>指定错误类型的错误条数/全部质检错误条数，用于观察错误结构。</t>
         </is>
       </c>
     </row>
@@ -2050,27 +2050,10 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>错误类型占比</t>
+          <t>新用户错误占比</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
-        <is>
-          <t>指定错误类型的错误条数/全部质检错误条数，用于观察错误结构。</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>新用户错误占比</t>
-        </is>
-      </c>
-      <c r="C92" s="3" t="inlineStr">
         <is>
           <t>新用户产生的质检错误条数/全部质检错误条数；新用户口径需按平台注册或首单时间窗统一定义。</t>
         </is>

</xml_diff>

<commit_message>
Remove task quality module
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1804,261 +1804,20 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="52" customHeight="1">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>进行中任务数</t>
-        </is>
-      </c>
-      <c r="C77" s="3" t="inlineStr">
-        <is>
-          <t>截至所选统计期末状态为进行中且可被执行或提交的任务数量，按任务 ID 去重。</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="52" customHeight="1">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>参与人数</t>
-        </is>
-      </c>
-      <c r="C78" s="3" t="inlineStr">
-        <is>
-          <t>所选统计时间内产生领取、进入任务、提交或质检相关有效任务行为的去重用户数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="52" customHeight="1">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>提交量</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="inlineStr">
-        <is>
-          <t>所选统计时间内任务提交数据条数，同一数据多次提交按提交记录累计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="52" customHeight="1">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>标注质检通过率</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="inlineStr">
-        <is>
-          <t>所选统计时间内，标注任务中质检通过的数据条数/标注任务中已完成质检的数据条数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="52" customHeight="1">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>返工率</t>
-        </is>
-      </c>
-      <c r="C81" s="3" t="inlineStr">
-        <is>
-          <t>所选统计时间内，被退回或要求返修的数据条数/已质检或已提交的数据条数，按业务选择同一口径。</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="52" customHeight="1">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>人均日产能</t>
-        </is>
-      </c>
-      <c r="C82" s="3" t="inlineStr">
-        <is>
-          <t>所选统计日期的任务提交数据条数/同一统计日期有有效任务行为的去重用户数；选择周、月或近 N 天时建议展示区间日均。</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="52" customHeight="1">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>采集质检通过率</t>
-        </is>
-      </c>
-      <c r="C83" s="3" t="inlineStr">
-        <is>
-          <t>所选统计时间内，采集任务中质检通过的数据条数/采集任务中已完成质检的数据条数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="52" customHeight="1">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>数据产出趋势</t>
-        </is>
-      </c>
-      <c r="C84" s="3" t="inlineStr">
-        <is>
-          <t>按日期展示标注提交数据条数和采集提交数据条数，用于观察不同任务类型的数据产出变化。</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="52" customHeight="1">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>标注提交数据条数</t>
-        </is>
-      </c>
-      <c r="C85" s="3" t="inlineStr">
-        <is>
-          <t>所选统计时间内标注任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="52" customHeight="1">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>采集提交数据条数</t>
-        </is>
-      </c>
-      <c r="C86" s="3" t="inlineStr">
-        <is>
-          <t>所选统计时间内采集任务产生的提交数据条数，同一数据多次提交按提交记录累计。</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="52" customHeight="1">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>后续质检通过率趋势</t>
-        </is>
-      </c>
-      <c r="C87" s="3" t="inlineStr">
-        <is>
-          <t>按日期展示后续质检通过率；后续质检通过率为首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数，不拆分具体轮次。</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="52" customHeight="1">
-      <c r="A88" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>后续质检通过率</t>
-        </is>
-      </c>
-      <c r="C88" s="3" t="inlineStr">
-        <is>
-          <t>首次质检未通过后在后续质检中通过的数据条数/进入后续质检并完成检查的数据条数；不拆分具体轮次。</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="52" customHeight="1">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
-        <is>
-          <t>错误类型分布</t>
-        </is>
-      </c>
-      <c r="C89" s="3" t="inlineStr">
-        <is>
-          <t>按错误类型展示质检错误结构，错误类型占比为指定错误类型的错误条数/全部质检错误条数。</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="15" customHeight="1">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>错误类型占比</t>
-        </is>
-      </c>
-      <c r="C90" s="3" t="inlineStr">
-        <is>
-          <t>指定错误类型的错误条数/全部质检错误条数，用于观察错误结构。</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>任务&amp;质量</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>新用户错误占比</t>
-        </is>
-      </c>
-      <c r="C91" s="3" t="inlineStr">
-        <is>
-          <t>新用户产生的质检错误条数/全部质检错误条数；新用户口径需按平台注册或首单时间窗统一定义。</t>
-        </is>
-      </c>
-    </row>
+    <row r="77" ht="52" customHeight="1"/>
+    <row r="78" ht="52" customHeight="1"/>
+    <row r="79" ht="52" customHeight="1"/>
+    <row r="80" ht="52" customHeight="1"/>
+    <row r="81" ht="52" customHeight="1"/>
+    <row r="82" ht="52" customHeight="1"/>
+    <row r="83" ht="52" customHeight="1"/>
+    <row r="84" ht="52" customHeight="1"/>
+    <row r="85" ht="52" customHeight="1"/>
+    <row r="86" ht="52" customHeight="1"/>
+    <row r="87" ht="52" customHeight="1"/>
+    <row r="88" ht="52" customHeight="1"/>
+    <row r="89" ht="52" customHeight="1"/>
+    <row r="90" ht="15" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:C92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Restore registration filters for churn and lifecycle
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -1375,7 +1375,7 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>暂不提供筛选，按当前样本截至 T+1 最新统计日观察相邻转化环节的流失人数和流失率；不展示跨环节平均流失率，不等同于 90 天未活跃或已流失用户。</t>
+          <t>支持筛选用户注册时间，筛选的是该时间范围内新注册的用户；观察这批用户截至昨日在相邻转化环节的流失人数和流失率，不展示跨环节平均流失率。</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>当前样本用户截至 T+1 最新统计日进入指定环节后未进入下一环节的去重用户数；与转化环节流失率使用同一批进入该环节的用户作为基准。</t>
+          <t>当前样本用户截至 T+1 最新统计日进入指定环节后未进入下一环节的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1409,7 @@
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>当前样本用户截至 T+1 最新统计日进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数；用于比较相邻转化断点，不应对多个环节简单平均，不等同于 90 天未活跃或已流失用户。</t>
+          <t>当前样本用户截至 T+1 最新统计日进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数。</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>当前样本用户截至 T+1 最新统计日流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位最明显的转化阻塞点。</t>
+          <t>所选用户注册时间内新注册用户中，截至 T+1 最新统计日流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位最明显的转化阻塞点。</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>暂不提供筛选，按当前样本截至 T+1 最新统计日观察用户从注册到流失判定或统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
+          <t>支持筛选用户注册时间，筛选的是该时间范围内新注册的用户；统计这批用户截至昨日从注册到流失判定或统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>当前样本用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到 T+1 最新统计日，已流失按连续 90 天无登录且无有效任务行为判定。</t>
+          <t>所选用户注册时间内新注册用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到 T+1 最新统计日，已流失按连续 90 天无登录且无有效任务行为判定。</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1477,7 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>当前样本用户从完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
+          <t>所选用户注册时间内新注册用户从完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到 T+1 最新统计日。</t>
+          <t>所选用户注册时间内新注册用户中，生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到 T+1 最新统计日。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove registration conversion metric
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -877,12 +877,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>新访客注册转化率</t>
+          <t>实名认证率</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>核心指标时间内首次访问平台的新访客中，截至该统计期末完成注册的新访客数/同一核心指标时间内首次访问平台的新访客数；时间筛选的是新访客首次访问时间。</t>
+          <t>核心指标时间内注册且截至该统计期末已完成实名认证的用户数/同一核心指标时间内具备实名认证资格的注册用户数；时间筛选的是用户注册时间，未开始认证和认证失败均不计入已认证用户数。</t>
         </is>
       </c>
     </row>
@@ -894,12 +894,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>实名认证率</t>
+          <t>招募申请率</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>核心指标时间内注册且截至该统计期末已完成实名认证的用户数/同一核心指标时间内具备实名认证资格的注册用户数；时间筛选的是用户注册时间，未开始认证和认证失败均不计入已认证用户数。</t>
+          <t>核心指标时间内注册且截至该统计期末完成实名认证后提交过至少一次招募申请的用户数/同一核心指标时间内完成实名认证且可申请招募的用户数；时间筛选的是用户注册时间。</t>
         </is>
       </c>
     </row>
@@ -911,12 +911,12 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>招募申请率</t>
+          <t>用户增长趋势</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>核心指标时间内注册且截至该统计期末完成实名认证后提交过至少一次招募申请的用户数/同一核心指标时间内完成实名认证且可申请招募的用户数；时间筛选的是用户注册时间。</t>
+          <t>固定展示近 7 日趋势，时间口径为事件发生日；每日展示新增注册、活跃用户和首次达到 90 天未活跃的用户变化。</t>
         </is>
       </c>
     </row>
@@ -928,12 +928,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>用户增长趋势</t>
+          <t>新用户转化漏斗</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>固定展示近 7 日趋势，时间口径为事件发生日；每日展示新增注册、活跃用户和首次达到 90 天未活跃的用户变化。</t>
+          <t>与用户留存矩阵联动，时间口径为留存矩阵中选定的注册周；展示该批新用户截至 T+1 最新统计日到达完成实名认证、提交招募申请、招募通过和首次任务执行等阶段的人数。</t>
         </is>
       </c>
     </row>
@@ -945,12 +945,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>新用户转化漏斗</t>
+          <t>新注册用户</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>与用户留存矩阵联动，时间口径为留存矩阵中选定的注册周；展示该批新用户截至 T+1 最新统计日到达完成实名认证、提交招募申请、招募通过和首次任务执行等阶段的人数。</t>
+          <t>留存矩阵中选定注册周内完成注册的去重用户数，是新用户转化漏斗和留存矩阵联动分析的基准用户数。</t>
         </is>
       </c>
     </row>
@@ -962,12 +962,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>新注册用户</t>
+          <t>完成实名认证</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>留存矩阵中选定注册周内完成注册的去重用户数，是新用户转化漏斗和留存矩阵联动分析的基准用户数。</t>
+          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日已完成实名认证的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -979,12 +979,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>完成实名认证</t>
+          <t>提交招募申请</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日已完成实名认证的去重用户数。</t>
+          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日至少提交过一次招募申请的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -996,12 +996,12 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>提交招募申请</t>
+          <t>招募通过</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日至少提交过一次招募申请的去重用户数。</t>
+          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日至少有一个招募申请审核通过的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1013,12 +1013,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>招募通过</t>
+          <t>首次任务执行</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日至少有一个招募申请审核通过的去重用户数。</t>
+          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日已产生首次有效任务行为的去重用户数；有效任务行为建议优先使用首次有效任务提交。</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1030,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>首次任务执行</t>
+          <t>环节转化率</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>留存矩阵中选定注册周用户里，截至 T+1 最新统计日已产生首次有效任务行为的去重用户数；有效任务行为建议优先使用首次有效任务提交。</t>
+          <t>当前阶段达成人数/上一阶段达成人数；首个阶段按 100% 展示。</t>
         </is>
       </c>
     </row>
@@ -1047,12 +1047,12 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>环节转化率</t>
+          <t>累计转化率</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>当前阶段达成人数/上一阶段达成人数；首个阶段按 100% 展示。</t>
+          <t>当前阶段达成人数/该漏斗入组的新注册用户数。</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>累计转化率</t>
+          <t>较上一步流失</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>当前阶段达成人数/该漏斗入组的新注册用户数。</t>
+          <t>上一阶段达成人数减去当前阶段达成人数，用于识别相邻阶段掉队规模。</t>
         </is>
       </c>
     </row>
@@ -1081,12 +1081,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>较上一步流失</t>
+          <t>用户留存矩阵（按注册周）</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>上一阶段达成人数减去当前阶段达成人数，用于识别相邻阶段掉队规模。</t>
+          <t>只提供周数筛选，用于选择近 N 个注册周；按注册周分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率，点击某一注册周可同步查看该批新用户的当前转化漏斗。</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>用户留存矩阵（按注册周）</t>
+          <t>注册分组用户数</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>只提供周数筛选，用于选择近 N 个注册周；按注册周分组展示用户在注册后 D1、D7、D14、D30 的活跃留存率，点击某一注册周可同步查看该批新用户的当前转化漏斗。</t>
+          <t>留存矩阵按近 N 个注册周筛选，指定注册周内完成注册的去重用户数，是 D1/D7/D14/D30 留存率的基准用户数。</t>
         </is>
       </c>
     </row>
@@ -1115,12 +1115,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>注册分组用户数</t>
+          <t>D1 留存</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>留存矩阵按近 N 个注册周筛选，指定注册周内完成注册的去重用户数，是 D1/D7/D14/D30 留存率的基准用户数。</t>
+          <t>指定注册周期用户中注册后第 1 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
@@ -1132,12 +1132,12 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>D1 留存</t>
+          <t>D7 留存</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>指定注册周期用户中注册后第 1 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
+          <t>指定注册周期用户中注册后第 7 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
@@ -1149,12 +1149,12 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>D7 留存</t>
+          <t>D14 留存</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>指定注册周期用户中注册后第 7 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
+          <t>指定注册周期用户中注册后第 14 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>D14 留存</t>
+          <t>D30 留存</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>指定注册周期用户中注册后第 14 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
+          <t>指定注册周期用户中注册后第 30 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
         </is>
       </c>
     </row>
@@ -1183,12 +1183,12 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>D30 留存</t>
+          <t>用户生命周期阶段分布</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>指定注册周期用户中注册后第 30 天仍有登录、访问核心页面或有效任务行为的用户数/该注册周期用户数。</t>
+          <t>不提供时间筛选，按 T+1 最新统计日快照统计用户最新生命周期状态；各阶段占比按该阶段用户数/注册总用户数计算，各阶段互斥统计。</t>
         </is>
       </c>
     </row>
@@ -1200,12 +1200,12 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>用户生命周期阶段分布</t>
+          <t>新注册</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>不提供时间筛选，按 T+1 最新统计日快照统计用户最新生命周期状态；各阶段占比按该阶段用户数/注册总用户数计算，各阶段互斥统计。</t>
+          <t>截至 T+1 最新统计日注册未满 7 天，且尚未进入实名认证、招募申请或任务执行阶段的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1217,12 +1217,12 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>新注册</t>
+          <t>待实名认证</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>截至 T+1 最新统计日注册未满 7 天，且尚未进入实名认证、招募申请或任务执行阶段的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日已完成注册但尚未完成实名认证，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1234,12 +1234,12 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>待实名认证</t>
+          <t>未申请过招募</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>截至 T+1 最新统计日已完成注册但尚未完成实名认证，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日已完成实名认证但从未提交招募申请，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1251,12 +1251,12 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>未申请过招募</t>
+          <t>招募审核中</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>截至 T+1 最新统计日已完成实名认证但从未提交招募申请，且未被判定为 30 日未活跃、60 日沉睡或已流失的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日至少提交过一次招募申请，且最新有效申请仍处于待审核或审核中状态的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1268,12 +1268,12 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>招募审核中</t>
+          <t>招募申请通过</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>截至 T+1 最新统计日至少提交过一次招募申请，且最新有效申请仍处于待审核或审核中状态的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日至少有一个招募申请已审核通过，但尚未产生有效任务执行行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1285,12 +1285,12 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>招募申请通过</t>
+          <t>活跃执行中</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>截至 T+1 最新统计日至少有一个招募申请已审核通过，但尚未产生有效任务执行行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日近 30 天内有有效任务领取、进入任务、提交或质检相关行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1302,12 +1302,12 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>活跃执行中</t>
+          <t>30日未活跃</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>截至 T+1 最新统计日近 30 天内有有效任务领取、进入任务、提交或质检相关行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日连续 30 天无登录且无有效任务行为，但尚未达到 60 天沉睡或 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1319,12 +1319,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>30日未活跃</t>
+          <t>60日沉睡</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>截至 T+1 最新统计日连续 30 天无登录且无有效任务行为，但尚未达到 60 天沉睡或 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日连续 60 天无登录且无有效任务行为，但尚未达到 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
         </is>
       </c>
     </row>
@@ -1336,12 +1336,12 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>60日沉睡</t>
+          <t>已流失用户</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>截至 T+1 最新统计日连续 60 天无登录且无有效任务行为，但尚未达到 90 天已流失标准的去重用户数；图中占比按该阶段用户数/注册总用户数计算。</t>
+          <t>截至 T+1 最新统计日连续 90 天无登录且无有效任务行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算，重新登录或产生有效任务行为后退出已流失状态。</t>
         </is>
       </c>
     </row>
@@ -1353,12 +1353,12 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>已流失用户</t>
+          <t>转化流失断点分析</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>截至 T+1 最新统计日连续 90 天无登录且无有效任务行为的去重用户数；图中占比按该阶段用户数/注册总用户数计算，重新登录或产生有效任务行为后退出已流失状态。</t>
+          <t>支持筛选用户注册时间，筛选的是该时间范围内新注册的用户；观察这批用户截至昨日在相邻转化环节的流失人数和流失率，不展示跨环节平均流失率。</t>
         </is>
       </c>
     </row>
@@ -1370,12 +1370,12 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>转化流失断点分析</t>
+          <t>转化环节流失人数</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>支持筛选用户注册时间，筛选的是该时间范围内新注册的用户；观察这批用户截至昨日在相邻转化环节的流失人数和流失率，不展示跨环节平均流失率。</t>
+          <t>当前样本用户截至 T+1 最新统计日进入指定环节后未进入下一环节的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1387,12 +1387,12 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>转化环节流失人数</t>
+          <t>转化环节流失率</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>当前样本用户截至 T+1 最新统计日进入指定环节后未进入下一环节的去重用户数。</t>
+          <t>当前样本用户截至 T+1 最新统计日进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数。</t>
         </is>
       </c>
     </row>
@@ -1404,12 +1404,12 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>转化环节流失率</t>
+          <t>最大流失断点</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>当前样本用户截至 T+1 最新统计日进入指定转化环节后未进入下一环节的用户数/进入该环节的用户数。</t>
+          <t>所选用户注册时间内新注册用户中，截至 T+1 最新统计日流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位最明显的转化阻塞点。</t>
         </is>
       </c>
     </row>
@@ -1421,12 +1421,12 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>最大流失断点</t>
+          <t>用户平均生命周期时长</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>所选用户注册时间内新注册用户中，截至 T+1 最新统计日流失率最高的转化环节，同时展示该环节未进入下一环节的用户数；用于定位最明显的转化阻塞点。</t>
+          <t>支持筛选用户注册时间，筛选的是该时间范围内新注册的用户；统计这批用户截至昨日从注册到流失判定或统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
         </is>
       </c>
     </row>
@@ -1438,12 +1438,12 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>用户平均生命周期时长</t>
+          <t>平均生命周期</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>支持筛选用户注册时间，筛选的是该时间范围内新注册的用户；统计这批用户截至昨日从注册到流失判定或统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
+          <t>所选用户注册时间内新注册用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到 T+1 最新统计日，已流失按连续 90 天无登录且无有效任务行为判定。</t>
         </is>
       </c>
     </row>
@@ -1455,12 +1455,12 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>平均生命周期</t>
+          <t>注册→首单</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>所选用户注册时间内新注册用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到 T+1 最新统计日，已流失按连续 90 天无登录且无有效任务行为判定。</t>
+          <t>所选用户注册时间内新注册用户从完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
         </is>
       </c>
     </row>
@@ -1472,29 +1472,29 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>注册→首单</t>
+          <t>生命周期时长分布</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>所选用户注册时间内新注册用户从完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
+          <t>所选用户注册时间内新注册用户中，生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到 T+1 最新统计日。</t>
         </is>
       </c>
     </row>
     <row r="58" ht="52" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>增长&amp;留存</t>
+          <t>招募分析</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>生命周期时长分布</t>
+          <t>新增招募单</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>所选用户注册时间内新注册用户中，生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到 T+1 最新统计日。</t>
+          <t>统计日新创建，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；统计日为 T+1 最新可用日期，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1506,12 +1506,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>新增招募单</t>
+          <t>进行中招募单</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>统计日新创建，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；统计日为 T+1 最新可用日期，默认与前一统计日对比。</t>
+          <t>统计日当前状态为招募中、仍可接收用户申请，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1523,12 +1523,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>进行中招募单</t>
+          <t>已完成招募单</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>统计日当前状态为招募中、仍可接收用户申请，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；默认与前一统计日对比。</t>
+          <t>统计日状态变更为已完成，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1540,12 +1540,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>已完成招募单</t>
+          <t>目标招募总人数</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>统计日状态变更为已完成，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成，默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1557,12 +1557,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>目标招募总人数</t>
+          <t>招募通过总人数</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>招募通过总人数</t>
+          <t>总缺口人数</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1591,12 +1591,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>总缺口人数</t>
+          <t>整体通过率</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1608,12 +1608,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>整体通过率</t>
+          <t>招募转化趋势</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，默认与前一统计日对比。</t>
+          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示申请率和通过率趋势。</t>
         </is>
       </c>
     </row>
@@ -1625,12 +1625,12 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>招募转化趋势</t>
+          <t>申请率</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示申请率和通过率趋势。</t>
+          <t>所选趋势时间内，符合当前领域筛选的提交招募申请去重用户数/访问或曝光该招募单且具备申请资格的去重用户数；招募指标卡片默认按统计日与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1642,12 +1642,12 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>申请率</t>
+          <t>通过率</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>所选趋势时间内，符合当前领域筛选的提交招募申请去重用户数/访问或曝光该招募单且具备申请资格的去重用户数；招募指标卡片默认按统计日与前一统计日对比。</t>
+          <t>所选趋势时间内，符合当前领域筛选的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，招募指标卡片默认按统计日与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1659,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>通过率</t>
+          <t>招募单数</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>所选趋势时间内，符合当前领域筛选的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，招募指标卡片默认按统计日与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1676,12 +1676,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>招募单数</t>
+          <t>目标人数</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量，默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1693,12 +1693,12 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>目标人数</t>
+          <t>申请人数</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1710,12 +1710,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>申请人数</t>
+          <t>招募通过人数</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次；默认与前一统计日对比。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1727,12 +1727,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>招募通过人数</t>
+          <t>缺口人数</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1744,12 +1744,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>缺口人数</t>
+          <t>缺口率</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的缺口人数/目标招募人数；目标人数为 0 时不计算，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1761,12 +1761,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>缺口率</t>
+          <t>平均审核周期</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的缺口人数/目标招募人数；目标人数为 0 时不计算，默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围、已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1778,32 +1778,16 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>平均审核周期</t>
+          <t>明细招募单状态</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围、已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计；默认与前一统计日对比。</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="52" customHeight="1">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>明细招募单状态</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
           <t>明细招募单在统计日的当前状态，包含招募中、审核中、已暂停、已完成，用于配合招募单状态筛选查看不同状态下的招募表现。</t>
         </is>
       </c>
     </row>
+    <row r="76" ht="52" customHeight="1"/>
     <row r="77" ht="52" customHeight="1"/>
     <row r="78" ht="52" customHeight="1"/>
     <row r="79" ht="52" customHeight="1"/>

</xml_diff>

<commit_message>
Update recruitment metric definitions and trend chart
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -1596,7 +1596,7 @@
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，默认与前一统计日对比。</t>
+          <t>所选时间范围内，截止对应日期招募审核通过人数/（招募审核通过+招募审核拒绝人数）；统计范围为当前领域与招募单状态筛选后的招募单集合。</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示申请率和通过率趋势。</t>
+          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示申请人数、申请率和通过率趋势。</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>所选趋势时间内，符合当前领域筛选的提交招募申请去重用户数/访问或曝光该招募单且具备申请资格的去重用户数；招募指标卡片默认按统计日与前一统计日对比。</t>
+          <t>所选时间范围内，当日提交招募申请去重用户数/当日访问该招募单的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1647,7 +1647,7 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>所选趋势时间内，符合当前领域筛选的审核通过招募申请数/已完成审核招募申请数；待审核申请不纳入计算，招募指标卡片默认按统计日与前一统计日对比。</t>
+          <t>所选时间范围内，截止对应日期招募审核通过人数/（招募审核通过+招募审核拒绝人数）。</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、提交过招募申请的去重用户数，同一用户对同一招募单多次申请只计一次；默认与前一统计日对比。</t>
+          <t>所选时间范围内，当日提交招募申请的去重用户数。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Unify recruitment trend metrics to cumulative definitions
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -1613,7 +1613,7 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示申请人数、申请率和通过率趋势。</t>
+          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示累计申请人数、累计申请率和累计通过率趋势。</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内，当日提交招募申请去重用户数/当日访问该招募单的去重用户数。</t>
+          <t>所选时间范围内，截止对应日期累计提交招募申请去重用户数/截止对应日期累计访问该招募单的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内，当日提交招募申请的去重用户数。</t>
+          <t>所选时间范围内，截止对应日期累计提交招募申请的去重用户数。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Split daily applications trend from recruitment conversion trend
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示累计申请人数、累计申请率和累计通过率趋势。</t>
+          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示累计申请率和累计通过率趋势。</t>
         </is>
       </c>
     </row>
@@ -1698,24 +1698,24 @@
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内，截止对应日期累计提交招募申请的去重用户数。</t>
+          <t>所选时间范围内，当日提交招募申请的去重用户数。</t>
         </is>
       </c>
     </row>
     <row r="71" ht="52" customHeight="1">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="A71" t="inlineStr">
         <is>
           <t>招募分析</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>招募通过人数</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>每日申请人数趋势</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>支持独立趋势时间筛选，筛选的是申请发生时间；按日期展示当日提交招募申请的去重用户数变化。</t>
         </is>
       </c>
     </row>
@@ -1727,12 +1727,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>缺口人数</t>
+          <t>招募通过人数</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1744,12 +1744,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>缺口率</t>
+          <t>缺口人数</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的缺口人数/目标招募人数；目标人数为 0 时不计算，默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1761,12 +1761,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>平均审核周期</t>
+          <t>缺口率</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围、已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的缺口人数/目标招募人数；目标人数为 0 时不计算，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1778,16 +1778,32 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
+          <t>平均审核周期</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>统计日符合当前领域与招募单状态筛选范围、已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计；默认与前一统计日对比。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="52" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>招募分析</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
           <t>明细招募单状态</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>明细招募单在统计日的当前状态，包含招募中、审核中、已暂停、已完成，用于配合招募单状态筛选查看不同状态下的招募表现。</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="52" customHeight="1"/>
     <row r="77" ht="52" customHeight="1"/>
     <row r="78" ht="52" customHeight="1"/>
     <row r="79" ht="52" customHeight="1"/>

</xml_diff>

<commit_message>
Remove lifecycle duration module
</commit_message>
<xml_diff>
--- a/docs/众包运营数据看板指标说明_最新发布版.xlsx
+++ b/docs/众包运营数据看板指标说明_最新发布版.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1416,68 +1416,68 @@
     <row r="54" ht="52" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>增长&amp;留存</t>
+          <t>招募分析</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>用户平均生命周期时长</t>
+          <t>新增招募单</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>支持筛选用户注册时间，筛选的是该时间范围内新注册的用户；统计这批用户截至昨日从注册到流失判定或统计期末的生命周期时长，并展示平均生命周期、注册到首单时长和时长区间分布。</t>
+          <t>统计日新创建，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；统计日为 T+1 最新可用日期，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
     <row r="55" ht="52" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>增长&amp;留存</t>
+          <t>招募分析</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>平均生命周期</t>
+          <t>进行中招募单</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>所选用户注册时间内新注册用户从注册到已流失判定日的平均天数；未达到已流失状态的用户统计到 T+1 最新统计日，已流失按连续 90 天无登录且无有效任务行为判定。</t>
+          <t>统计日当前状态为招募中、仍可接收用户申请，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
     <row r="56" ht="52" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>增长&amp;留存</t>
+          <t>招募分析</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>注册→首单</t>
+          <t>已完成招募单</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>所选用户注册时间内新注册用户从完成注册到首次产生有效任务行为之间的平均时长，有效任务行为可包括领取、进入任务或首次提交。</t>
+          <t>统计日状态变更为已完成，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
     <row r="57" ht="52" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>增长&amp;留存</t>
+          <t>招募分析</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>生命周期时长分布</t>
+          <t>目标招募总人数</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>所选用户注册时间内新注册用户中，生命周期时长落入指定区间的用户数/纳入生命周期统计的用户总数；生命周期时长从注册日统计到已流失判定日，未流失用户统计到 T+1 最新统计日。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1489,12 +1489,12 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>新增招募单</t>
+          <t>招募通过总人数</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>统计日新创建，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；统计日为 T+1 最新可用日期，默认与前一统计日对比。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1506,12 +1506,12 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>进行中招募单</t>
+          <t>总缺口人数</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>统计日当前状态为招募中、仍可接收用户申请，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1523,12 +1523,12 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>已完成招募单</t>
+          <t>整体通过率</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>统计日状态变更为已完成，且符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；关闭或暂停不等同于完成，默认与前一统计日对比。</t>
+          <t>所选时间范围内，截止对应日期招募审核通过人数/（招募审核通过+招募审核拒绝人数）；统计范围为当前领域与招募单状态筛选后的招募单集合。</t>
         </is>
       </c>
     </row>
@@ -1540,12 +1540,12 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>目标招募总人数</t>
+          <t>招募转化趋势</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
+          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示累计申请率和累计通过率趋势。</t>
         </is>
       </c>
     </row>
@@ -1557,12 +1557,12 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>招募通过总人数</t>
+          <t>申请率</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
+          <t>所选时间范围内，截止对应日期累计提交招募申请去重用户数/截止对应日期累计访问该招募单的去重用户数。</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1574,12 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>总缺口人数</t>
+          <t>通过率</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
+          <t>所选时间范围内，截止对应日期招募审核通过人数/（招募审核通过+招募审核拒绝人数）。</t>
         </is>
       </c>
     </row>
@@ -1591,12 +1591,12 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>整体通过率</t>
+          <t>招募单数</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内，截止对应日期招募审核通过人数/（招募审核通过+招募审核拒绝人数）；统计范围为当前领域与招募单状态筛选后的招募单集合。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1608,12 +1608,12 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>招募转化趋势</t>
+          <t>目标人数</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>支持独立趋势时间筛选，筛选的是申请或审核发生时间；按日期展示累计申请率和累计通过率趋势。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1625,29 +1625,29 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>申请率</t>
+          <t>申请人数</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内，截止对应日期累计提交招募申请去重用户数/截止对应日期累计访问该招募单的去重用户数。</t>
+          <t>所选时间范围内，当日提交招募申请的去重用户数。</t>
         </is>
       </c>
     </row>
     <row r="67" ht="52" customHeight="1">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>通过率</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>所选时间范围内，截止对应日期招募审核通过人数/（招募审核通过+招募审核拒绝人数）。</t>
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>招募分析</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>每日申请人数趋势</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>支持独立趋势时间筛选，筛选的是申请发生时间；按日期展示当日提交招募申请的去重用户数变化。</t>
         </is>
       </c>
     </row>
@@ -1659,12 +1659,12 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>招募单数</t>
+          <t>招募通过人数</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的招募单数量，按招募单 ID 去重；按领域查看时表示该领域下的招募单数量，默认与前一统计日对比。</t>
+          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1676,12 +1676,12 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>目标人数</t>
+          <t>缺口人数</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的招募单计划招募人数合计，按招募单目标人数汇总；默认与前一统计日对比。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1693,29 +1693,29 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>申请人数</t>
+          <t>缺口率</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>所选时间范围内，当日提交招募申请的去重用户数。</t>
+          <t>统计日符合当前领域与招募单状态筛选范围的缺口人数/目标招募人数；目标人数为 0 时不计算，默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
     <row r="71" ht="52" customHeight="1">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>每日申请人数趋势</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>支持独立趋势时间筛选，筛选的是申请发生时间；按日期展示当日提交招募申请的去重用户数变化。</t>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>招募分析</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>平均审核周期</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>统计日符合当前领域与招募单状态筛选范围、已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计；默认与前一统计日对比。</t>
         </is>
       </c>
     </row>
@@ -1727,83 +1727,19 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>招募通过人数</t>
+          <t>明细招募单状态</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>统计日累计符合当前领域与招募单状态筛选范围、招募申请审核通过的去重用户数，同一用户在同一招募单只计一次；默认与前一统计日对比。</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="52" customHeight="1">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>缺口人数</t>
-        </is>
-      </c>
-      <c r="C73" s="3" t="inlineStr">
-        <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的目标招募人数减去招募通过人数后的缺口人数，结果小于 0 时按 0 统计；默认与前一统计日对比。</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="52" customHeight="1">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>缺口率</t>
-        </is>
-      </c>
-      <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>统计日符合当前领域与招募单状态筛选范围的缺口人数/目标招募人数；目标人数为 0 时不计算，默认与前一统计日对比。</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="52" customHeight="1">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>平均审核周期</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="inlineStr">
-        <is>
-          <t>统计日符合当前领域与招募单状态筛选范围、已完成审核的申请从提交申请到审批完成的平均时长，待审核申请不纳入统计；默认与前一统计日对比。</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="52" customHeight="1">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>招募分析</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>明细招募单状态</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
           <t>明细招募单在统计日的当前状态，包含招募中、审核中、已暂停、已完成，用于配合招募单状态筛选查看不同状态下的招募表现。</t>
         </is>
       </c>
     </row>
+    <row r="73" ht="52" customHeight="1"/>
+    <row r="74" ht="52" customHeight="1"/>
+    <row r="75" ht="52" customHeight="1"/>
+    <row r="76" ht="52" customHeight="1"/>
     <row r="77" ht="52" customHeight="1"/>
     <row r="78" ht="52" customHeight="1"/>
     <row r="79" ht="52" customHeight="1"/>

</xml_diff>